<commit_message>
fixed hrremainstype and aircontainertype
</commit_message>
<xml_diff>
--- a/CargoUIAutomationNew/src/test/resources/TestCasesMapping.xlsx
+++ b/CargoUIAutomationNew/src/test/resources/TestCasesMapping.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26731"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26924"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\LocalFiles\p57448\CargoUIAutomation\src\test\resources\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\workspace\IdeaProjects\Cargo\CargoUIAutomationNew\src\test\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EFFA5690-8281-4F34-806F-F4CECC87A91A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7F9805FD-A080-4DF8-80C8-2BFA470AB6C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" firstSheet="1" activeTab="2" xr2:uid="{1AB005B2-AFEC-3B46-93EF-50FA3BE3C5FF}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="11" activeTab="18" xr2:uid="{1AB005B2-AFEC-3B46-93EF-50FA3BE3C5FF}"/>
   </bookViews>
   <sheets>
     <sheet name="Configuration" sheetId="14" r:id="rId1"/>
@@ -40,32 +40,24 @@
     <definedName name="DataColumnRange">MasterSheet!$A$2:$A$129</definedName>
     <definedName name="dataRowRange">MasterSheet!$B$1:$AL$1</definedName>
   </definedNames>
-  <calcPr calcId="191028"/>
+  <calcPr calcId="181029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <metadataTypes count="1">
     <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
   </metadataTypes>
   <futureMetadata name="XLDAPR" count="1">
     <bk>
       <extLst>
-        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
+        <ext xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray" uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
           <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
         </ext>
       </extLst>
@@ -80,7 +72,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5270" uniqueCount="409">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5271" uniqueCount="409">
   <si>
     <t>LoginCredentials</t>
   </si>
@@ -1313,9 +1305,16 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="11">
+  <fonts count="12">
     <font>
       <sz val="12"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -1640,9 +1639,9 @@
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="75">
+  <cellXfs count="76">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
@@ -1650,25 +1649,25 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
@@ -1676,25 +1675,25 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" quotePrefix="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="2" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="2" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="9" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1704,14 +1703,14 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1720,46 +1719,46 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="9" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="9" fillId="4" borderId="1" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="10" fillId="4" borderId="1" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1768,7 +1767,7 @@
     <xf numFmtId="49" fontId="0" fillId="4" borderId="1" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" quotePrefix="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1819,21 +1818,21 @@
     <xf numFmtId="0" fontId="0" fillId="14" borderId="1" xfId="0" quotePrefix="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="17" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="18" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="19" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="20" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="21" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="22" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="17" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="18" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="19" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="20" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="21" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="22" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="22" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="22" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="23" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="23" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="23" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="23" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1841,6 +1840,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" quotePrefix="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -2165,12 +2167,12 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FA4D241A-A8EF-49D1-8679-699235E5685A}">
   <sheetPr codeName="Sheet1"/>
   <dimension ref="A1:C5"/>
-  <sheetFormatPr defaultColWidth="8.83203125" defaultRowHeight="15.5"/>
+  <sheetFormatPr defaultColWidth="8.796875" defaultRowHeight="15.6"/>
   <cols>
-    <col min="1" max="1" width="32.83203125" style="11" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="32.796875" style="11" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="31" style="11" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="25" style="11" bestFit="1" customWidth="1"/>
-    <col min="4" max="16384" width="8.83203125" style="11"/>
+    <col min="4" max="16384" width="8.796875" style="11"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -2240,16 +2242,16 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A0B29DB4-834B-3D43-AE5D-83E0EA72CBB8}">
   <dimension ref="A1:AL15"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.5"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.6"/>
   <cols>
     <col min="1" max="1" width="101" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="16" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="27.58203125" customWidth="1"/>
+    <col min="3" max="3" width="27.59765625" customWidth="1"/>
     <col min="9" max="9" width="14" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="18.5" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="15.33203125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="15.296875" bestFit="1" customWidth="1"/>
     <col min="37" max="37" width="11.5" bestFit="1" customWidth="1"/>
-    <col min="38" max="38" width="17.58203125" customWidth="1"/>
+    <col min="38" max="38" width="17.59765625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:38" s="11" customFormat="1">
@@ -2368,7 +2370,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="2" spans="1:38" ht="16.5">
+    <row r="2" spans="1:38" ht="16.8">
       <c r="A2" s="32" t="s">
         <v>278</v>
       </c>
@@ -2519,7 +2521,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="3" spans="1:38" ht="16.5">
+    <row r="3" spans="1:38" ht="16.8">
       <c r="A3" s="32" t="s">
         <v>279</v>
       </c>
@@ -2670,7 +2672,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="4" spans="1:38" ht="16.5">
+    <row r="4" spans="1:38" ht="16.8">
       <c r="A4" s="32" t="s">
         <v>280</v>
       </c>
@@ -2821,7 +2823,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="5" spans="1:38" ht="16.5">
+    <row r="5" spans="1:38" ht="16.8">
       <c r="A5" s="32" t="s">
         <v>281</v>
       </c>
@@ -2972,7 +2974,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="6" spans="1:38" ht="16.5">
+    <row r="6" spans="1:38" ht="16.8">
       <c r="A6" s="32" t="s">
         <v>282</v>
       </c>
@@ -3123,7 +3125,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="7" spans="1:38" ht="16.5">
+    <row r="7" spans="1:38" ht="16.8">
       <c r="A7" s="32" t="s">
         <v>283</v>
       </c>
@@ -3274,7 +3276,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="8" spans="1:38" ht="16.5">
+    <row r="8" spans="1:38" ht="16.8">
       <c r="A8" s="32" t="s">
         <v>284</v>
       </c>
@@ -3425,7 +3427,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="9" spans="1:38" ht="16.5">
+    <row r="9" spans="1:38" ht="16.8">
       <c r="A9" s="32" t="s">
         <v>285</v>
       </c>
@@ -3576,7 +3578,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="10" spans="1:38" ht="16.5">
+    <row r="10" spans="1:38" ht="16.8">
       <c r="A10" s="32" t="s">
         <v>286</v>
       </c>
@@ -3727,7 +3729,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="11" spans="1:38" ht="16.5">
+    <row r="11" spans="1:38" ht="16.8">
       <c r="A11" s="32" t="s">
         <v>287</v>
       </c>
@@ -3878,7 +3880,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="12" spans="1:38" ht="16.5">
+    <row r="12" spans="1:38" ht="16.8">
       <c r="A12" s="32" t="s">
         <v>288</v>
       </c>
@@ -4029,7 +4031,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="13" spans="1:38" ht="16.5">
+    <row r="13" spans="1:38" ht="16.8">
       <c r="A13" s="32" t="s">
         <v>289</v>
       </c>
@@ -4180,7 +4182,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="14" spans="1:38" ht="16.5">
+    <row r="14" spans="1:38" ht="16.8">
       <c r="A14" s="32" t="s">
         <v>290</v>
       </c>
@@ -4331,7 +4333,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="15" spans="1:38" ht="16.5">
+    <row r="15" spans="1:38" ht="16.8">
       <c r="A15" s="32" t="s">
         <v>291</v>
       </c>
@@ -4495,18 +4497,18 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7508C757-379C-BD45-982F-A9AA36397E0D}">
   <dimension ref="A1:Z36"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.5"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.6"/>
   <cols>
-    <col min="1" max="1" width="51.83203125" customWidth="1"/>
+    <col min="1" max="1" width="51.796875" customWidth="1"/>
     <col min="2" max="2" width="14.5" customWidth="1"/>
     <col min="3" max="3" width="25.5" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="14.83203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14.796875" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="41" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="37.08203125" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="20.08203125" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="22.08203125" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="27.08203125" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="7.83203125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="37.09765625" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="20.09765625" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="22.09765625" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="27.09765625" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="7.796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:26">
@@ -7119,49 +7121,49 @@
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2E6A7DA2-FEB7-B54D-86C6-DFEA37D68DD1}">
   <dimension ref="A1:AM7"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.5"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.6"/>
   <cols>
     <col min="1" max="1" width="102" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="16" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="23.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="23.296875" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="9" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="14.58203125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="23.83203125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="13.33203125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="14.83203125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="18.83203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="14.59765625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="23.796875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13.296875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="14.796875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="18.796875" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="14" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="18.5" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="15.58203125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="18.33203125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="15.59765625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="18.296875" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="15" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="19.5" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="16" bestFit="1" customWidth="1"/>
     <col min="17" max="17" width="14.5" bestFit="1" customWidth="1"/>
     <col min="18" max="18" width="14" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="14.33203125" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="14.296875" bestFit="1" customWidth="1"/>
     <col min="20" max="20" width="12.5" bestFit="1" customWidth="1"/>
     <col min="21" max="21" width="19" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="25.33203125" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="37.08203125" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="21.58203125" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="20.08203125" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="25.296875" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="37.09765625" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="21.59765625" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="20.09765625" bestFit="1" customWidth="1"/>
     <col min="26" max="26" width="28" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="12.83203125" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="32.33203125" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="22.08203125" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="24.08203125" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="29.08203125" customWidth="1"/>
-    <col min="32" max="33" width="8.58203125" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="4.08203125" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="12.796875" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="32.296875" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="22.09765625" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="24.09765625" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="29.09765625" customWidth="1"/>
+    <col min="32" max="33" width="8.59765625" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="4.09765625" bestFit="1" customWidth="1"/>
     <col min="35" max="35" width="5.5" bestFit="1" customWidth="1"/>
-    <col min="36" max="36" width="6.08203125" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="14.33203125" bestFit="1" customWidth="1"/>
-    <col min="38" max="38" width="14.33203125" customWidth="1"/>
-    <col min="39" max="39" width="21.08203125" customWidth="1"/>
+    <col min="36" max="36" width="6.09765625" bestFit="1" customWidth="1"/>
+    <col min="37" max="37" width="14.296875" bestFit="1" customWidth="1"/>
+    <col min="38" max="38" width="14.296875" customWidth="1"/>
+    <col min="39" max="39" width="21.09765625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:39" s="11" customFormat="1" ht="16" thickBot="1">
+    <row r="1" spans="1:39" s="11" customFormat="1" ht="16.2" thickBot="1">
       <c r="A1" s="19" t="s">
         <v>118</v>
       </c>
@@ -7280,7 +7282,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="2" spans="1:39" ht="17" thickBot="1">
+    <row r="2" spans="1:39" ht="17.399999999999999" thickBot="1">
       <c r="A2" s="64" t="s">
         <v>306</v>
       </c>
@@ -7435,7 +7437,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:39" ht="17" thickBot="1">
+    <row r="3" spans="1:39" ht="17.399999999999999" thickBot="1">
       <c r="A3" s="64" t="s">
         <v>307</v>
       </c>
@@ -7590,7 +7592,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:39" ht="17" thickBot="1">
+    <row r="4" spans="1:39" ht="17.399999999999999" thickBot="1">
       <c r="A4" s="64" t="s">
         <v>308</v>
       </c>
@@ -7745,7 +7747,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:39" ht="17" thickBot="1">
+    <row r="5" spans="1:39" ht="17.399999999999999" thickBot="1">
       <c r="A5" s="64" t="s">
         <v>309</v>
       </c>
@@ -7900,7 +7902,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:39" ht="17" thickBot="1">
+    <row r="6" spans="1:39" ht="17.399999999999999" thickBot="1">
       <c r="A6" s="64" t="s">
         <v>310</v>
       </c>
@@ -8055,7 +8057,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:39" ht="17" thickBot="1">
+    <row r="7" spans="1:39" ht="17.399999999999999" thickBot="1">
       <c r="A7" s="64" t="s">
         <v>311</v>
       </c>
@@ -8221,18 +8223,18 @@
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{78402954-2B6D-C042-9263-9F192091C8D5}">
   <dimension ref="A1:AN7"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.5"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.6"/>
   <cols>
-    <col min="1" max="1" width="62.83203125" customWidth="1"/>
+    <col min="1" max="1" width="62.796875" customWidth="1"/>
     <col min="2" max="2" width="16" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="23.08203125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="14.58203125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="23.83203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="23.09765625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="14.59765625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="23.796875" bestFit="1" customWidth="1"/>
     <col min="38" max="38" width="16" customWidth="1"/>
-    <col min="40" max="40" width="13.33203125" customWidth="1"/>
+    <col min="40" max="40" width="13.296875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:40" s="11" customFormat="1" ht="16" thickBot="1">
+    <row r="1" spans="1:40" s="11" customFormat="1" ht="16.2" thickBot="1">
       <c r="A1" s="19" t="s">
         <v>118</v>
       </c>
@@ -8354,7 +8356,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="2" spans="1:40" ht="17" thickBot="1">
+    <row r="2" spans="1:40" ht="17.399999999999999" thickBot="1">
       <c r="A2" s="65" t="s">
         <v>302</v>
       </c>
@@ -8513,7 +8515,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:40" ht="17" thickBot="1">
+    <row r="3" spans="1:40" ht="17.399999999999999" thickBot="1">
       <c r="A3" s="65" t="s">
         <v>303</v>
       </c>
@@ -8672,7 +8674,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="1:40" ht="17" thickBot="1">
+    <row r="4" spans="1:40" ht="17.399999999999999" thickBot="1">
       <c r="A4" s="65" t="s">
         <v>304</v>
       </c>
@@ -8831,7 +8833,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="5" spans="1:40" ht="17" thickBot="1">
+    <row r="5" spans="1:40" ht="17.399999999999999" thickBot="1">
       <c r="A5" s="65" t="s">
         <v>305</v>
       </c>
@@ -8990,7 +8992,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="6" spans="1:40" ht="17" thickBot="1">
+    <row r="6" spans="1:40" ht="17.399999999999999" thickBot="1">
       <c r="A6" s="65" t="s">
         <v>398</v>
       </c>
@@ -9149,7 +9151,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="7" spans="1:40" ht="17" thickBot="1">
+    <row r="7" spans="1:40" ht="17.399999999999999" thickBot="1">
       <c r="A7" s="65" t="s">
         <v>399</v>
       </c>
@@ -9319,48 +9321,48 @@
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D85CBF01-6F2F-C544-96AC-B46CDE75B137}">
   <dimension ref="A1:AL13"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.5"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.6"/>
   <cols>
-    <col min="1" max="1" width="89.25" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="89.19921875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="16" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="23" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="8.83203125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="23.58203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="8.796875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="23.59765625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="13" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.25" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14.19921875" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="19" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.75" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="18.33203125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="18.08203125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="18.25" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="14.58203125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="13.69921875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="18.296875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="18.09765625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="18.19921875" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="14.59765625" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="19" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="16" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="14.33203125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="13.83203125" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="14.08203125" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="12.08203125" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="18.75" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="25.08203125" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="37.08203125" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="21.25" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="20.08203125" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="14.296875" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="13.796875" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="14.09765625" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="12.09765625" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="18.69921875" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="25.09765625" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="37.09765625" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="21.19921875" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="20.09765625" bestFit="1" customWidth="1"/>
     <col min="25" max="25" width="28" bestFit="1" customWidth="1"/>
     <col min="26" max="26" width="13" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="32.25" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="21.58203125" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="22.83203125" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="13.33203125" bestFit="1" customWidth="1"/>
-    <col min="31" max="32" width="8.25" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="6.25" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="6.58203125" bestFit="1" customWidth="1"/>
-    <col min="35" max="35" width="5.75" bestFit="1" customWidth="1"/>
-    <col min="36" max="36" width="14.33203125" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="32.19921875" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="21.59765625" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="22.796875" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="13.296875" bestFit="1" customWidth="1"/>
+    <col min="31" max="32" width="8.19921875" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="6.19921875" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="6.59765625" bestFit="1" customWidth="1"/>
+    <col min="35" max="35" width="5.69921875" bestFit="1" customWidth="1"/>
+    <col min="36" max="36" width="14.296875" bestFit="1" customWidth="1"/>
     <col min="37" max="37" width="11.5" bestFit="1" customWidth="1"/>
-    <col min="38" max="38" width="4.75" bestFit="1" customWidth="1"/>
+    <col min="38" max="38" width="4.69921875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:38" s="11" customFormat="1" ht="16" thickBot="1">
+    <row r="1" spans="1:38" s="11" customFormat="1" ht="16.2" thickBot="1">
       <c r="A1" s="19" t="s">
         <v>118</v>
       </c>
@@ -9476,7 +9478,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="2" spans="1:38" ht="17" thickBot="1">
+    <row r="2" spans="1:38" ht="17.399999999999999" thickBot="1">
       <c r="A2" s="69" t="s">
         <v>375</v>
       </c>
@@ -9627,7 +9629,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:38" ht="17" thickBot="1">
+    <row r="3" spans="1:38" ht="17.399999999999999" thickBot="1">
       <c r="A3" s="70" t="s">
         <v>376</v>
       </c>
@@ -9778,7 +9780,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:38" ht="17" thickBot="1">
+    <row r="4" spans="1:38" ht="17.399999999999999" thickBot="1">
       <c r="A4" s="70" t="s">
         <v>377</v>
       </c>
@@ -9929,7 +9931,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:38" ht="17" thickBot="1">
+    <row r="5" spans="1:38" ht="17.399999999999999" thickBot="1">
       <c r="A5" s="70" t="s">
         <v>378</v>
       </c>
@@ -10080,7 +10082,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:38" ht="17" thickBot="1">
+    <row r="6" spans="1:38" ht="17.399999999999999" thickBot="1">
       <c r="A6" s="70" t="s">
         <v>379</v>
       </c>
@@ -10231,7 +10233,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:38" ht="17" thickBot="1">
+    <row r="7" spans="1:38" ht="17.399999999999999" thickBot="1">
       <c r="A7" s="70" t="s">
         <v>380</v>
       </c>
@@ -10382,7 +10384,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:38" ht="17" thickBot="1">
+    <row r="8" spans="1:38" ht="17.399999999999999" thickBot="1">
       <c r="A8" s="70" t="s">
         <v>381</v>
       </c>
@@ -10533,7 +10535,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:38" ht="17" thickBot="1">
+    <row r="9" spans="1:38" ht="17.399999999999999" thickBot="1">
       <c r="A9" s="70" t="s">
         <v>382</v>
       </c>
@@ -10684,7 +10686,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:38" ht="17" thickBot="1">
+    <row r="10" spans="1:38" ht="17.399999999999999" thickBot="1">
       <c r="A10" s="70" t="s">
         <v>383</v>
       </c>
@@ -10835,7 +10837,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:38" ht="17" thickBot="1">
+    <row r="11" spans="1:38" ht="17.399999999999999" thickBot="1">
       <c r="A11" s="70" t="s">
         <v>384</v>
       </c>
@@ -10986,7 +10988,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:38" ht="17" thickBot="1">
+    <row r="12" spans="1:38" ht="17.399999999999999" thickBot="1">
       <c r="A12" s="70" t="s">
         <v>385</v>
       </c>
@@ -11137,7 +11139,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:38" ht="17" thickBot="1">
+    <row r="13" spans="1:38" ht="17.399999999999999" thickBot="1">
       <c r="A13" s="70" t="s">
         <v>386</v>
       </c>
@@ -11300,19 +11302,19 @@
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EFFF123C-E07E-C740-AE81-4E891CD59C3F}">
   <dimension ref="A1:AM11"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.5"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.6"/>
   <cols>
-    <col min="1" max="1" width="92.58203125" customWidth="1"/>
-    <col min="3" max="3" width="46.08203125" customWidth="1"/>
-    <col min="4" max="4" width="8.75" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="14.58203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="92.59765625" customWidth="1"/>
+    <col min="3" max="3" width="46.09765625" customWidth="1"/>
+    <col min="4" max="4" width="8.69921875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="14.59765625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="25" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="42.58203125" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="20.08203125" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="22.08203125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="42.59765625" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="20.09765625" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="22.09765625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:39" s="11" customFormat="1" ht="16" thickBot="1">
+    <row r="1" spans="1:39" s="11" customFormat="1" ht="16.2" thickBot="1">
       <c r="A1" s="19" t="s">
         <v>118</v>
       </c>
@@ -11431,7 +11433,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="2" spans="1:39" ht="17" thickBot="1">
+    <row r="2" spans="1:39" ht="17.399999999999999" thickBot="1">
       <c r="A2" t="s">
         <v>388</v>
       </c>
@@ -11586,7 +11588,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:39" ht="17" thickBot="1">
+    <row r="3" spans="1:39" ht="17.399999999999999" thickBot="1">
       <c r="A3" t="s">
         <v>389</v>
       </c>
@@ -11741,7 +11743,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:39" ht="17" thickBot="1">
+    <row r="4" spans="1:39" ht="17.399999999999999" thickBot="1">
       <c r="A4" t="s">
         <v>390</v>
       </c>
@@ -11896,7 +11898,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:39" ht="17" thickBot="1">
+    <row r="5" spans="1:39" ht="17.399999999999999" thickBot="1">
       <c r="A5" t="s">
         <v>391</v>
       </c>
@@ -12051,7 +12053,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:39" ht="17" thickBot="1">
+    <row r="6" spans="1:39" ht="17.399999999999999" thickBot="1">
       <c r="A6" t="s">
         <v>392</v>
       </c>
@@ -12206,7 +12208,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:39" ht="17" thickBot="1">
+    <row r="7" spans="1:39" ht="17.399999999999999" thickBot="1">
       <c r="A7" t="s">
         <v>393</v>
       </c>
@@ -12361,7 +12363,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:39" ht="17" thickBot="1">
+    <row r="8" spans="1:39" ht="17.399999999999999" thickBot="1">
       <c r="A8" t="s">
         <v>394</v>
       </c>
@@ -12516,7 +12518,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:39" ht="17" thickBot="1">
+    <row r="9" spans="1:39" ht="17.399999999999999" thickBot="1">
       <c r="A9" t="s">
         <v>395</v>
       </c>
@@ -12671,7 +12673,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:39" ht="17" thickBot="1">
+    <row r="10" spans="1:39" ht="17.399999999999999" thickBot="1">
       <c r="A10" t="s">
         <v>396</v>
       </c>
@@ -12826,7 +12828,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:39" ht="17" thickBot="1">
+    <row r="11" spans="1:39" ht="17.399999999999999" thickBot="1">
       <c r="A11" t="s">
         <v>397</v>
       </c>
@@ -12993,18 +12995,18 @@
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A9B20742-2F64-BB4D-931D-0ED7AB74219D}">
   <dimension ref="A1:AM11"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.5"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.6"/>
   <cols>
-    <col min="1" max="1" width="158.58203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="57.58203125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="14.58203125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="22.08203125" customWidth="1"/>
+    <col min="1" max="1" width="158.59765625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="57.59765625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="14.59765625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="22.09765625" customWidth="1"/>
     <col min="7" max="7" width="24.5" customWidth="1"/>
-    <col min="11" max="11" width="8.75" customWidth="1"/>
-    <col min="12" max="12" width="47.33203125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="8.69921875" customWidth="1"/>
+    <col min="12" max="12" width="47.296875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:39" s="11" customFormat="1" ht="16" thickBot="1">
+    <row r="1" spans="1:39" s="11" customFormat="1" ht="16.2" thickBot="1">
       <c r="A1" s="19" t="s">
         <v>118</v>
       </c>
@@ -13123,7 +13125,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="2" spans="1:39" ht="17" thickBot="1">
+    <row r="2" spans="1:39" ht="17.399999999999999" thickBot="1">
       <c r="A2" s="66" t="s">
         <v>338</v>
       </c>
@@ -13278,7 +13280,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:39" ht="17" thickBot="1">
+    <row r="3" spans="1:39" ht="17.399999999999999" thickBot="1">
       <c r="A3" s="66" t="s">
         <v>339</v>
       </c>
@@ -13433,7 +13435,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:39" ht="17" thickBot="1">
+    <row r="4" spans="1:39" ht="17.399999999999999" thickBot="1">
       <c r="A4" s="66" t="s">
         <v>340</v>
       </c>
@@ -13588,7 +13590,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:39" ht="17" thickBot="1">
+    <row r="5" spans="1:39" ht="17.399999999999999" thickBot="1">
       <c r="A5" s="66" t="s">
         <v>341</v>
       </c>
@@ -13743,7 +13745,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:39" ht="17" thickBot="1">
+    <row r="6" spans="1:39" ht="17.399999999999999" thickBot="1">
       <c r="A6" s="66" t="s">
         <v>342</v>
       </c>
@@ -13898,7 +13900,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:39" ht="17" thickBot="1">
+    <row r="7" spans="1:39" ht="17.399999999999999" thickBot="1">
       <c r="A7" s="66" t="s">
         <v>343</v>
       </c>
@@ -14053,7 +14055,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:39" ht="17" thickBot="1">
+    <row r="8" spans="1:39" ht="17.399999999999999" thickBot="1">
       <c r="A8" s="66" t="s">
         <v>344</v>
       </c>
@@ -14208,7 +14210,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:39" ht="17" thickBot="1">
+    <row r="9" spans="1:39" ht="17.399999999999999" thickBot="1">
       <c r="A9" s="66" t="s">
         <v>345</v>
       </c>
@@ -14363,7 +14365,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:39" ht="17" thickBot="1">
+    <row r="10" spans="1:39" ht="17.399999999999999" thickBot="1">
       <c r="A10" s="66" t="s">
         <v>346</v>
       </c>
@@ -14518,7 +14520,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:39" ht="17" thickBot="1">
+    <row r="11" spans="1:39" ht="17.399999999999999" thickBot="1">
       <c r="A11" s="66" t="s">
         <v>347</v>
       </c>
@@ -14685,15 +14687,15 @@
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{22440E3A-6E10-F44C-A8EB-A92A916ABD32}">
   <dimension ref="A1:AL13"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.5"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.6"/>
   <cols>
     <col min="1" max="1" width="128.5" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15.58203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.59765625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="55.5" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="23.83203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="23.796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:38" s="11" customFormat="1" ht="16" thickBot="1">
+    <row r="1" spans="1:38" s="11" customFormat="1" ht="16.2" thickBot="1">
       <c r="A1" s="19" t="s">
         <v>118</v>
       </c>
@@ -14809,7 +14811,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="2" spans="1:38" ht="17" thickBot="1">
+    <row r="2" spans="1:38" ht="17.399999999999999" thickBot="1">
       <c r="A2" s="67" t="s">
         <v>348</v>
       </c>
@@ -14960,7 +14962,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:38" ht="17" thickBot="1">
+    <row r="3" spans="1:38" ht="17.399999999999999" thickBot="1">
       <c r="A3" s="67" t="s">
         <v>349</v>
       </c>
@@ -15111,7 +15113,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:38" ht="17" thickBot="1">
+    <row r="4" spans="1:38" ht="17.399999999999999" thickBot="1">
       <c r="A4" s="67" t="s">
         <v>350</v>
       </c>
@@ -15262,7 +15264,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:38" ht="17" thickBot="1">
+    <row r="5" spans="1:38" ht="17.399999999999999" thickBot="1">
       <c r="A5" s="67" t="s">
         <v>351</v>
       </c>
@@ -15413,7 +15415,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:38" ht="17" thickBot="1">
+    <row r="6" spans="1:38" ht="17.399999999999999" thickBot="1">
       <c r="A6" s="67" t="s">
         <v>352</v>
       </c>
@@ -15564,7 +15566,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:38" ht="17" thickBot="1">
+    <row r="7" spans="1:38" ht="17.399999999999999" thickBot="1">
       <c r="A7" s="67" t="s">
         <v>353</v>
       </c>
@@ -15715,7 +15717,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:38" ht="17" thickBot="1">
+    <row r="8" spans="1:38" ht="17.399999999999999" thickBot="1">
       <c r="A8" s="67" t="s">
         <v>354</v>
       </c>
@@ -15866,7 +15868,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:38" ht="17" thickBot="1">
+    <row r="9" spans="1:38" ht="17.399999999999999" thickBot="1">
       <c r="A9" s="67" t="s">
         <v>355</v>
       </c>
@@ -16017,7 +16019,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:38" ht="17" thickBot="1">
+    <row r="10" spans="1:38" ht="17.399999999999999" thickBot="1">
       <c r="A10" s="67" t="s">
         <v>356</v>
       </c>
@@ -16168,7 +16170,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:38" ht="17" thickBot="1">
+    <row r="11" spans="1:38" ht="17.399999999999999" thickBot="1">
       <c r="A11" s="67" t="s">
         <v>357</v>
       </c>
@@ -16319,7 +16321,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:38" ht="17" thickBot="1">
+    <row r="12" spans="1:38" ht="17.399999999999999" thickBot="1">
       <c r="A12" s="67" t="s">
         <v>358</v>
       </c>
@@ -16470,7 +16472,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:38" ht="17" thickBot="1">
+    <row r="13" spans="1:38" ht="17.399999999999999" thickBot="1">
       <c r="A13" s="67" t="s">
         <v>359</v>
       </c>
@@ -16632,14 +16634,14 @@
 <file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EA53CA9E-5475-8E48-80D6-77CE99F7CA3D}">
   <dimension ref="A1:AM5"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.5"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.6"/>
   <cols>
-    <col min="1" max="1" width="114.58203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="114.59765625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="22.5" bestFit="1" customWidth="1"/>
-    <col min="5" max="6" width="14.58203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="6" width="14.59765625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:39" s="11" customFormat="1" ht="16" thickBot="1">
+    <row r="1" spans="1:39" s="11" customFormat="1" ht="16.2" thickBot="1">
       <c r="A1" s="19" t="s">
         <v>118</v>
       </c>
@@ -16758,7 +16760,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="2" spans="1:39" ht="16" thickBot="1">
+    <row r="2" spans="1:39" ht="16.2" thickBot="1">
       <c r="A2" s="68" t="s">
         <v>360</v>
       </c>
@@ -16913,7 +16915,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:39" ht="16" thickBot="1">
+    <row r="3" spans="1:39" ht="16.2" thickBot="1">
       <c r="A3" s="68" t="s">
         <v>361</v>
       </c>
@@ -17068,7 +17070,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:39" ht="16" thickBot="1">
+    <row r="4" spans="1:39" ht="16.2" thickBot="1">
       <c r="A4" s="68" t="s">
         <v>400</v>
       </c>
@@ -17223,7 +17225,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:39" ht="16" thickBot="1">
+    <row r="5" spans="1:39" ht="16.2" thickBot="1">
       <c r="A5" s="68" t="s">
         <v>401</v>
       </c>
@@ -17393,15 +17395,15 @@
 <file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{35458118-D48A-D94F-8815-70903938F945}">
   <dimension ref="A1:AM7"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.5"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.6"/>
   <cols>
     <col min="1" max="1" width="105" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="17.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="23.33203125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="14.58203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="23.296875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="14.59765625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:39" s="11" customFormat="1" ht="16" thickBot="1">
+    <row r="1" spans="1:39" s="11" customFormat="1" ht="16.2" thickBot="1">
       <c r="A1" s="19" t="s">
         <v>118</v>
       </c>
@@ -17520,7 +17522,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="2" spans="1:39" ht="16" thickBot="1">
+    <row r="2" spans="1:39" ht="16.2" thickBot="1">
       <c r="A2" s="71" t="s">
         <v>403</v>
       </c>
@@ -17558,9 +17560,8 @@
         <f t="array" ref="J2">_xlfn.XLOOKUP($A2,DataColumnRange,_xlfn.XLOOKUP(J$1,dataRowRange,ActualDataRange))</f>
         <v>ATL</v>
       </c>
-      <c r="K2" s="31" t="str" cm="1">
-        <f t="array" ref="K2">_xlfn.XLOOKUP($A2,DataColumnRange,_xlfn.XLOOKUP(K$1,dataRowRange,ActualDataRange))</f>
-        <v>MSP</v>
+      <c r="K2" s="75" t="s">
+        <v>143</v>
       </c>
       <c r="L2" s="31" t="str" cm="1">
         <f t="array" ref="L2">_xlfn.XLOOKUP($A2,DataColumnRange,_xlfn.XLOOKUP(L$1,dataRowRange,ActualDataRange))</f>
@@ -17675,7 +17676,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:39" ht="16" thickBot="1">
+    <row r="3" spans="1:39" ht="16.2" thickBot="1">
       <c r="A3" s="72" t="s">
         <v>404</v>
       </c>
@@ -17830,7 +17831,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:39" ht="16" thickBot="1">
+    <row r="4" spans="1:39" ht="16.2" thickBot="1">
       <c r="A4" s="72" t="s">
         <v>405</v>
       </c>
@@ -17985,7 +17986,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:39" ht="16" thickBot="1">
+    <row r="5" spans="1:39" ht="16.2" thickBot="1">
       <c r="A5" s="72" t="s">
         <v>406</v>
       </c>
@@ -18140,7 +18141,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:39" ht="16" thickBot="1">
+    <row r="6" spans="1:39" ht="16.2" thickBot="1">
       <c r="A6" s="72" t="s">
         <v>407</v>
       </c>
@@ -18295,7 +18296,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:39" ht="16" thickBot="1">
+    <row r="7" spans="1:39" ht="16.2" thickBot="1">
       <c r="A7" s="72" t="s">
         <v>408</v>
       </c>
@@ -18462,13 +18463,13 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FF8DD980-905D-FC4A-81AD-0000D690C0FF}">
   <sheetPr codeName="Sheet3"/>
   <dimension ref="A1:E16"/>
-  <sheetFormatPr defaultColWidth="10.83203125" defaultRowHeight="15.5"/>
+  <sheetFormatPr defaultColWidth="10.796875" defaultRowHeight="15.6"/>
   <cols>
-    <col min="1" max="1" width="47.58203125" style="11" customWidth="1"/>
-    <col min="2" max="3" width="16.58203125" style="11" customWidth="1"/>
-    <col min="4" max="4" width="10.83203125" style="11" customWidth="1"/>
+    <col min="1" max="1" width="47.59765625" style="11" customWidth="1"/>
+    <col min="2" max="3" width="16.59765625" style="11" customWidth="1"/>
+    <col min="4" max="4" width="10.796875" style="11" customWidth="1"/>
     <col min="5" max="5" width="31" style="11" customWidth="1"/>
-    <col min="6" max="16384" width="10.83203125" style="11"/>
+    <col min="6" max="16384" width="10.796875" style="11"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5">
@@ -18488,7 +18489,7 @@
         <v>273</v>
       </c>
     </row>
-    <row r="2" spans="1:5" ht="32.15" customHeight="1">
+    <row r="2" spans="1:5" ht="32.1" customHeight="1">
       <c r="A2" s="11" t="s">
         <v>139</v>
       </c>
@@ -18506,7 +18507,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:5" ht="16">
+    <row r="3" spans="1:5">
       <c r="A3" s="11" t="s">
         <v>138</v>
       </c>
@@ -18524,7 +18525,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:5" ht="16">
+    <row r="4" spans="1:5">
       <c r="A4" s="11" t="s">
         <v>167</v>
       </c>
@@ -18542,7 +18543,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="5" spans="1:5" ht="16">
+    <row r="5" spans="1:5">
       <c r="A5" s="11" t="s">
         <v>168</v>
       </c>
@@ -18560,7 +18561,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="6" spans="1:5" ht="16">
+    <row r="6" spans="1:5">
       <c r="A6" s="11" t="s">
         <v>169</v>
       </c>
@@ -18578,7 +18579,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="7" spans="1:5" ht="16">
+    <row r="7" spans="1:5">
       <c r="A7" s="11" t="s">
         <v>170</v>
       </c>
@@ -18596,7 +18597,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="8" spans="1:5" ht="16">
+    <row r="8" spans="1:5">
       <c r="A8" s="11" t="s">
         <v>199</v>
       </c>
@@ -18785,46 +18786,46 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1DAEE888-1773-9E47-9558-1F0A440779BF}">
   <dimension ref="A1:AL129"/>
-  <sheetFormatPr defaultColWidth="10.83203125" defaultRowHeight="15.5"/>
+  <sheetFormatPr defaultColWidth="10.796875" defaultRowHeight="15.6"/>
   <cols>
-    <col min="1" max="1" width="104.1640625" style="2" customWidth="1"/>
-    <col min="2" max="2" width="18.08203125" style="2" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="23.33203125" style="2" customWidth="1"/>
+    <col min="1" max="1" width="104.19921875" style="2" customWidth="1"/>
+    <col min="2" max="2" width="18.09765625" style="2" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="23.296875" style="2" customWidth="1"/>
     <col min="4" max="4" width="25.5" style="2" customWidth="1"/>
-    <col min="5" max="5" width="13.33203125" style="2" customWidth="1"/>
-    <col min="6" max="6" width="21.83203125" style="2" customWidth="1"/>
-    <col min="7" max="7" width="18.83203125" style="2" customWidth="1"/>
+    <col min="5" max="5" width="13.296875" style="2" customWidth="1"/>
+    <col min="6" max="6" width="21.796875" style="2" customWidth="1"/>
+    <col min="7" max="7" width="18.796875" style="2" customWidth="1"/>
     <col min="8" max="8" width="14" style="2" customWidth="1"/>
     <col min="9" max="9" width="18.5" style="2" customWidth="1"/>
     <col min="10" max="10" width="52" style="2" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="17.83203125" style="2" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="17.796875" style="2" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="15" style="2" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="19.5" style="2" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="16" style="2" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="14.5" style="2" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="14" style="2" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="14.33203125" style="2" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="14.296875" style="2" bestFit="1" customWidth="1"/>
     <col min="18" max="18" width="12.5" style="2" bestFit="1" customWidth="1"/>
     <col min="19" max="19" width="19" style="2" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="25.33203125" style="2" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="37.08203125" style="2" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="21.58203125" style="2" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="20.08203125" style="2" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="25.296875" style="2" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="37.09765625" style="2" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="21.59765625" style="2" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="20.09765625" style="2" bestFit="1" customWidth="1"/>
     <col min="24" max="24" width="28" style="2" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="10.83203125" style="2"/>
-    <col min="26" max="26" width="34.58203125" style="2" customWidth="1"/>
-    <col min="27" max="27" width="22.08203125" style="2" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="22.33203125" style="2" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="13.25" style="2" bestFit="1" customWidth="1"/>
-    <col min="30" max="31" width="8.58203125" style="2" bestFit="1" customWidth="1"/>
-    <col min="32" max="32" width="6.83203125" style="2" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="10.796875" style="2"/>
+    <col min="26" max="26" width="34.59765625" style="2" customWidth="1"/>
+    <col min="27" max="27" width="22.09765625" style="2" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="22.296875" style="2" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="13.19921875" style="2" bestFit="1" customWidth="1"/>
+    <col min="30" max="31" width="8.59765625" style="2" bestFit="1" customWidth="1"/>
+    <col min="32" max="32" width="6.796875" style="2" bestFit="1" customWidth="1"/>
     <col min="33" max="33" width="7.5" style="2" bestFit="1" customWidth="1"/>
     <col min="34" max="34" width="6" style="2" bestFit="1" customWidth="1"/>
-    <col min="35" max="35" width="14.33203125" style="2" bestFit="1" customWidth="1"/>
-    <col min="36" max="36" width="14.33203125" style="2" customWidth="1"/>
-    <col min="37" max="37" width="4.83203125" style="2" bestFit="1" customWidth="1"/>
-    <col min="38" max="38" width="16.58203125" style="2" customWidth="1"/>
-    <col min="39" max="16384" width="10.83203125" style="2"/>
+    <col min="35" max="35" width="14.296875" style="2" bestFit="1" customWidth="1"/>
+    <col min="36" max="36" width="14.296875" style="2" customWidth="1"/>
+    <col min="37" max="37" width="4.796875" style="2" bestFit="1" customWidth="1"/>
+    <col min="38" max="38" width="16.59765625" style="2" customWidth="1"/>
+    <col min="39" max="16384" width="10.796875" style="2"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:38">
@@ -33233,7 +33234,7 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:AL129" xr:uid="{1DAEE888-1773-9E47-9558-1F0A440779BF}"/>
-  <phoneticPr fontId="4" type="noConversion"/>
+  <phoneticPr fontId="5" type="noConversion"/>
   <hyperlinks>
     <hyperlink ref="D2" r:id="rId1" xr:uid="{A27DD8EB-70E3-9343-A2F0-4EC1F414F378}"/>
     <hyperlink ref="D3" r:id="rId2" xr:uid="{B7F22B40-D1E3-41A2-B580-43255BDF4D3A}"/>
@@ -33373,44 +33374,44 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{67F99C04-ED4A-B140-B723-3FB745556183}">
   <sheetPr codeName="Sheet4"/>
   <dimension ref="A1:AO7"/>
-  <sheetFormatPr defaultColWidth="10.83203125" defaultRowHeight="15.5"/>
+  <sheetFormatPr defaultColWidth="10.796875" defaultRowHeight="15.6"/>
   <cols>
     <col min="1" max="1" width="89.5" style="38" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="16" style="38" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="23.33203125" style="38" customWidth="1"/>
-    <col min="4" max="4" width="13.08203125" style="38" customWidth="1"/>
-    <col min="5" max="5" width="39.08203125" style="38" customWidth="1"/>
-    <col min="6" max="6" width="13.33203125" style="38" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.83203125" style="38" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="18.83203125" style="38" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="20.33203125" style="38" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="28.33203125" style="38" customWidth="1"/>
-    <col min="11" max="11" width="15.33203125" style="38" customWidth="1"/>
-    <col min="12" max="12" width="18.33203125" style="38" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="33.58203125" style="38" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="23.296875" style="38" customWidth="1"/>
+    <col min="4" max="4" width="13.09765625" style="38" customWidth="1"/>
+    <col min="5" max="5" width="39.09765625" style="38" customWidth="1"/>
+    <col min="6" max="6" width="13.296875" style="38" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14.796875" style="38" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="18.796875" style="38" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="20.296875" style="38" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="28.296875" style="38" customWidth="1"/>
+    <col min="11" max="11" width="15.296875" style="38" customWidth="1"/>
+    <col min="12" max="12" width="18.296875" style="38" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="33.59765625" style="38" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="19" style="38" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="25.33203125" style="38" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="37.08203125" style="38" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="21.58203125" style="38" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="20.08203125" style="38" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="25.296875" style="38" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="37.09765625" style="38" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="21.59765625" style="38" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="20.09765625" style="38" bestFit="1" customWidth="1"/>
     <col min="19" max="19" width="28" style="38" bestFit="1" customWidth="1"/>
     <col min="20" max="20" width="19" style="38" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="32.33203125" style="38" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="37.08203125" style="38" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="21.58203125" style="38" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="26.58203125" style="38" customWidth="1"/>
-    <col min="25" max="25" width="27.33203125" style="38" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="32.296875" style="38" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="37.09765625" style="38" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="21.59765625" style="38" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="26.59765625" style="38" customWidth="1"/>
+    <col min="25" max="25" width="27.296875" style="38" bestFit="1" customWidth="1"/>
     <col min="26" max="26" width="13" style="38" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="14.33203125" style="38" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="22.08203125" style="38" bestFit="1" customWidth="1"/>
-    <col min="29" max="35" width="10.83203125" style="38"/>
+    <col min="27" max="27" width="14.296875" style="38" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="22.09765625" style="38" bestFit="1" customWidth="1"/>
+    <col min="29" max="35" width="10.796875" style="38"/>
     <col min="36" max="36" width="14.5" style="38" bestFit="1" customWidth="1"/>
     <col min="37" max="37" width="14.5" style="38" customWidth="1"/>
-    <col min="38" max="38" width="10.83203125" style="38"/>
-    <col min="39" max="39" width="25.33203125" style="38" bestFit="1" customWidth="1"/>
-    <col min="40" max="40" width="37.08203125" style="38" bestFit="1" customWidth="1"/>
-    <col min="41" max="41" width="21.58203125" style="38" bestFit="1" customWidth="1"/>
-    <col min="42" max="16384" width="10.83203125" style="38"/>
+    <col min="38" max="38" width="10.796875" style="38"/>
+    <col min="39" max="39" width="25.296875" style="38" bestFit="1" customWidth="1"/>
+    <col min="40" max="40" width="37.09765625" style="38" bestFit="1" customWidth="1"/>
+    <col min="41" max="41" width="21.59765625" style="38" bestFit="1" customWidth="1"/>
+    <col min="42" max="16384" width="10.796875" style="38"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:41">
@@ -33538,7 +33539,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:41" ht="16">
+    <row r="2" spans="1:41">
       <c r="A2" s="39" t="s">
         <v>212</v>
       </c>
@@ -33701,7 +33702,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="3" spans="1:41" ht="16">
+    <row r="3" spans="1:41">
       <c r="A3" s="39" t="s">
         <v>213</v>
       </c>
@@ -33864,7 +33865,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="4" spans="1:41" ht="16">
+    <row r="4" spans="1:41">
       <c r="A4" s="39" t="s">
         <v>214</v>
       </c>
@@ -34028,7 +34029,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="5" spans="1:41" ht="16">
+    <row r="5" spans="1:41">
       <c r="A5" s="39" t="s">
         <v>217</v>
       </c>
@@ -34192,7 +34193,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="6" spans="1:41" ht="16">
+    <row r="6" spans="1:41">
       <c r="A6" s="39" t="s">
         <v>218</v>
       </c>
@@ -34356,7 +34357,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="7" spans="1:41" ht="16">
+    <row r="7" spans="1:41">
       <c r="A7" s="39" t="s">
         <v>219</v>
       </c>
@@ -34521,7 +34522,7 @@
       </c>
     </row>
   </sheetData>
-  <phoneticPr fontId="4" type="noConversion"/>
+  <phoneticPr fontId="5" type="noConversion"/>
   <hyperlinks>
     <hyperlink ref="D2" location="AdvBkngSTD!A1" display="AdvBkngSTD" xr:uid="{9836EF3A-0C81-384A-B28E-38769E19AD72}"/>
     <hyperlink ref="A1" location="TestCaseConfig!A1" display="TestCases" xr:uid="{B061C974-A2F8-7C4C-A5EC-974E6D31B128}"/>
@@ -34536,40 +34537,40 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6C996C58-3C8B-D941-9CF9-2A0431D4505C}">
   <sheetPr codeName="Sheet6"/>
   <dimension ref="A1:AL11"/>
-  <sheetFormatPr defaultColWidth="10.83203125" defaultRowHeight="15.5"/>
+  <sheetFormatPr defaultColWidth="10.796875" defaultRowHeight="15.6"/>
   <cols>
-    <col min="1" max="1" width="131.58203125" style="11" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="131.59765625" style="11" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="16" style="11" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="23.33203125" style="11" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10.83203125" style="11" customWidth="1"/>
+    <col min="3" max="3" width="23.296875" style="11" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.796875" style="11" customWidth="1"/>
     <col min="5" max="5" width="25.5" style="11" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="14.83203125" style="11" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="14.796875" style="11" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="19" style="11" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="20.33203125" style="11" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="20.296875" style="11" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="16" style="11" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="29" style="11" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="38.58203125" style="11" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="18.33203125" style="28" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="38.59765625" style="11" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="18.296875" style="28" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="15" style="11" bestFit="1" customWidth="1"/>
-    <col min="14" max="15" width="10.83203125" style="11"/>
-    <col min="16" max="16" width="21.58203125" style="11" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="20.08203125" style="11" bestFit="1" customWidth="1"/>
+    <col min="14" max="15" width="10.796875" style="11"/>
+    <col min="16" max="16" width="21.59765625" style="11" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="20.09765625" style="11" bestFit="1" customWidth="1"/>
     <col min="18" max="18" width="28" style="11" bestFit="1" customWidth="1"/>
     <col min="19" max="19" width="13" style="11" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="10.83203125" style="11"/>
-    <col min="21" max="21" width="22.08203125" style="11" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="22.83203125" style="11" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="13.58203125" style="11" bestFit="1" customWidth="1"/>
-    <col min="24" max="25" width="10.83203125" style="11"/>
-    <col min="26" max="26" width="14.33203125" style="11" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="38.58203125" style="11" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="22.08203125" style="11" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="22.83203125" style="11" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="13.58203125" style="11" bestFit="1" customWidth="1"/>
-    <col min="31" max="35" width="10.83203125" style="11"/>
-    <col min="36" max="36" width="14.33203125" style="11" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="14.33203125" style="11" customWidth="1"/>
-    <col min="38" max="16384" width="10.83203125" style="11"/>
+    <col min="20" max="20" width="10.796875" style="11"/>
+    <col min="21" max="21" width="22.09765625" style="11" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="22.796875" style="11" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="13.59765625" style="11" bestFit="1" customWidth="1"/>
+    <col min="24" max="25" width="10.796875" style="11"/>
+    <col min="26" max="26" width="14.296875" style="11" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="38.59765625" style="11" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="22.09765625" style="11" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="22.796875" style="11" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="13.59765625" style="11" bestFit="1" customWidth="1"/>
+    <col min="31" max="35" width="10.796875" style="11"/>
+    <col min="36" max="36" width="14.296875" style="11" bestFit="1" customWidth="1"/>
+    <col min="37" max="37" width="14.296875" style="11" customWidth="1"/>
+    <col min="38" max="16384" width="10.796875" style="11"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:38">
@@ -34688,7 +34689,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="2" spans="1:38" ht="16.5">
+    <row r="2" spans="1:38" ht="16.8">
       <c r="A2" s="33" t="s">
         <v>231</v>
       </c>
@@ -34839,7 +34840,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="3" spans="1:38" ht="16.5">
+    <row r="3" spans="1:38" ht="16.8">
       <c r="A3" s="33" t="s">
         <v>232</v>
       </c>
@@ -34990,7 +34991,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="4" spans="1:38" ht="16.5">
+    <row r="4" spans="1:38" ht="16.8">
       <c r="A4" s="33" t="s">
         <v>233</v>
       </c>
@@ -35141,7 +35142,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="5" spans="1:38" ht="16.5">
+    <row r="5" spans="1:38" ht="16.8">
       <c r="A5" s="33" t="s">
         <v>234</v>
       </c>
@@ -35292,7 +35293,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="6" spans="1:38" ht="16.5">
+    <row r="6" spans="1:38" ht="16.8">
       <c r="A6" s="33" t="s">
         <v>235</v>
       </c>
@@ -35443,7 +35444,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="7" spans="1:38" ht="16.5">
+    <row r="7" spans="1:38" ht="16.8">
       <c r="A7" s="33" t="s">
         <v>236</v>
       </c>
@@ -35594,7 +35595,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="8" spans="1:38" ht="16.5">
+    <row r="8" spans="1:38" ht="16.8">
       <c r="A8" s="33" t="s">
         <v>237</v>
       </c>
@@ -35745,7 +35746,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="9" spans="1:38" ht="16.5">
+    <row r="9" spans="1:38" ht="16.8">
       <c r="A9" s="33" t="s">
         <v>238</v>
       </c>
@@ -35896,7 +35897,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="10" spans="1:38" ht="16.5">
+    <row r="10" spans="1:38" ht="16.8">
       <c r="A10" s="33" t="s">
         <v>239</v>
       </c>
@@ -36047,7 +36048,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="11" spans="1:38" ht="16.5">
+    <row r="11" spans="1:38" ht="16.8">
       <c r="A11" s="33" t="s">
         <v>240</v>
       </c>
@@ -36213,17 +36214,17 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{63E70DB7-4DD6-624F-9EA1-30DDDFA58DD7}">
   <dimension ref="A1:AL11"/>
-  <sheetFormatPr defaultColWidth="10.83203125" defaultRowHeight="15.5"/>
+  <sheetFormatPr defaultColWidth="10.796875" defaultRowHeight="15.6"/>
   <cols>
-    <col min="1" max="1" width="145.33203125" style="11" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="145.296875" style="11" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="16" style="11" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="23.33203125" style="11" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="23.33203125" style="11" customWidth="1"/>
-    <col min="5" max="5" width="23.83203125" style="11" bestFit="1" customWidth="1"/>
-    <col min="6" max="10" width="10.83203125" style="11"/>
-    <col min="11" max="11" width="49.08203125" style="11" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="18.33203125" style="28" bestFit="1" customWidth="1"/>
-    <col min="13" max="16384" width="10.83203125" style="11"/>
+    <col min="3" max="3" width="23.296875" style="11" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="23.296875" style="11" customWidth="1"/>
+    <col min="5" max="5" width="23.796875" style="11" bestFit="1" customWidth="1"/>
+    <col min="6" max="10" width="10.796875" style="11"/>
+    <col min="11" max="11" width="49.09765625" style="11" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="18.296875" style="28" bestFit="1" customWidth="1"/>
+    <col min="13" max="16384" width="10.796875" style="11"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:38">
@@ -36342,7 +36343,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="2" spans="1:38" ht="16.5">
+    <row r="2" spans="1:38" ht="16.8">
       <c r="A2" s="33" t="s">
         <v>241</v>
       </c>
@@ -36493,7 +36494,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="3" spans="1:38" ht="16.5">
+    <row r="3" spans="1:38" ht="16.8">
       <c r="A3" s="33" t="s">
         <v>242</v>
       </c>
@@ -36644,7 +36645,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="4" spans="1:38" ht="16.5">
+    <row r="4" spans="1:38" ht="16.8">
       <c r="A4" s="33" t="s">
         <v>243</v>
       </c>
@@ -36795,7 +36796,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="5" spans="1:38" ht="16.5">
+    <row r="5" spans="1:38" ht="16.8">
       <c r="A5" s="33" t="s">
         <v>244</v>
       </c>
@@ -36946,7 +36947,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="6" spans="1:38" ht="16.5">
+    <row r="6" spans="1:38" ht="16.8">
       <c r="A6" s="33" t="s">
         <v>245</v>
       </c>
@@ -37097,7 +37098,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="7" spans="1:38" ht="16.5">
+    <row r="7" spans="1:38" ht="16.8">
       <c r="A7" s="33" t="s">
         <v>246</v>
       </c>
@@ -37248,7 +37249,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="8" spans="1:38" ht="16.5">
+    <row r="8" spans="1:38" ht="16.8">
       <c r="A8" s="33" t="s">
         <v>247</v>
       </c>
@@ -37399,7 +37400,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="9" spans="1:38" ht="16.5">
+    <row r="9" spans="1:38" ht="16.8">
       <c r="A9" s="33" t="s">
         <v>248</v>
       </c>
@@ -37550,7 +37551,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="10" spans="1:38" ht="16.5">
+    <row r="10" spans="1:38" ht="16.8">
       <c r="A10" s="33" t="s">
         <v>249</v>
       </c>
@@ -37701,7 +37702,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="11" spans="1:38" ht="16.5">
+    <row r="11" spans="1:38" ht="16.8">
       <c r="A11" s="33" t="s">
         <v>250</v>
       </c>
@@ -37866,16 +37867,16 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3E262B8C-B72A-DD49-A994-304B68688876}">
   <dimension ref="A1:AL13"/>
-  <sheetFormatPr defaultColWidth="10.83203125" defaultRowHeight="15.5"/>
+  <sheetFormatPr defaultColWidth="10.796875" defaultRowHeight="15.6"/>
   <cols>
     <col min="1" max="1" width="131.5" style="11" bestFit="1" customWidth="1"/>
-    <col min="2" max="3" width="10.83203125" style="11"/>
+    <col min="2" max="3" width="10.796875" style="11"/>
     <col min="4" max="4" width="13" style="11" customWidth="1"/>
-    <col min="5" max="5" width="23.83203125" style="11" bestFit="1" customWidth="1"/>
-    <col min="6" max="10" width="10.83203125" style="11"/>
-    <col min="11" max="11" width="47.33203125" style="11" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="18.33203125" style="28" bestFit="1" customWidth="1"/>
-    <col min="13" max="16384" width="10.83203125" style="11"/>
+    <col min="5" max="5" width="23.796875" style="11" bestFit="1" customWidth="1"/>
+    <col min="6" max="10" width="10.796875" style="11"/>
+    <col min="11" max="11" width="47.296875" style="11" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="18.296875" style="28" bestFit="1" customWidth="1"/>
+    <col min="13" max="16384" width="10.796875" style="11"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:38">
@@ -37994,7 +37995,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="2" spans="1:38" ht="16.5">
+    <row r="2" spans="1:38" ht="16.8">
       <c r="A2" s="32" t="s">
         <v>251</v>
       </c>
@@ -38145,7 +38146,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="3" spans="1:38" ht="16.5">
+    <row r="3" spans="1:38" ht="16.8">
       <c r="A3" s="32" t="s">
         <v>252</v>
       </c>
@@ -38296,7 +38297,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="4" spans="1:38" ht="16.5">
+    <row r="4" spans="1:38" ht="16.8">
       <c r="A4" s="32" t="s">
         <v>253</v>
       </c>
@@ -38447,7 +38448,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="5" spans="1:38" ht="16.5">
+    <row r="5" spans="1:38" ht="16.8">
       <c r="A5" s="32" t="s">
         <v>254</v>
       </c>
@@ -38598,7 +38599,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="6" spans="1:38" ht="16.5">
+    <row r="6" spans="1:38" ht="16.8">
       <c r="A6" s="32" t="s">
         <v>255</v>
       </c>
@@ -38749,7 +38750,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="7" spans="1:38" ht="16.5">
+    <row r="7" spans="1:38" ht="16.8">
       <c r="A7" s="32" t="s">
         <v>256</v>
       </c>
@@ -38900,7 +38901,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="8" spans="1:38" ht="16.5">
+    <row r="8" spans="1:38" ht="16.8">
       <c r="A8" s="32" t="s">
         <v>257</v>
       </c>
@@ -39051,7 +39052,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="9" spans="1:38" ht="16.5">
+    <row r="9" spans="1:38" ht="16.8">
       <c r="A9" s="32" t="s">
         <v>258</v>
       </c>
@@ -39202,7 +39203,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="10" spans="1:38" ht="16.5">
+    <row r="10" spans="1:38" ht="16.8">
       <c r="A10" s="32" t="s">
         <v>259</v>
       </c>
@@ -39353,7 +39354,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="11" spans="1:38" ht="16.5">
+    <row r="11" spans="1:38" ht="16.8">
       <c r="A11" s="32" t="s">
         <v>260</v>
       </c>
@@ -39504,7 +39505,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="12" spans="1:38" ht="16.5">
+    <row r="12" spans="1:38" ht="16.8">
       <c r="A12" s="32" t="s">
         <v>261</v>
       </c>
@@ -39655,7 +39656,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="13" spans="1:38" ht="16.5">
+    <row r="13" spans="1:38" ht="16.8">
       <c r="A13" s="32" t="s">
         <v>262</v>
       </c>
@@ -39820,17 +39821,17 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A7990930-FE48-954E-9FFC-70384FD7E025}">
   <dimension ref="A1:AL5"/>
-  <sheetFormatPr defaultColWidth="10.83203125" defaultRowHeight="15.5"/>
+  <sheetFormatPr defaultColWidth="10.796875" defaultRowHeight="15.6"/>
   <cols>
     <col min="1" max="1" width="102.5" style="11" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="16" style="11" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="23.33203125" style="11" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="25.58203125" style="11" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="23.83203125" style="11" bestFit="1" customWidth="1"/>
-    <col min="6" max="10" width="10.83203125" style="11"/>
+    <col min="3" max="3" width="23.296875" style="11" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="25.59765625" style="11" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="23.796875" style="11" bestFit="1" customWidth="1"/>
+    <col min="6" max="10" width="10.796875" style="11"/>
     <col min="11" max="11" width="24.5" style="11" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="18.33203125" style="28" bestFit="1" customWidth="1"/>
-    <col min="13" max="16384" width="10.83203125" style="11"/>
+    <col min="12" max="12" width="18.296875" style="28" bestFit="1" customWidth="1"/>
+    <col min="13" max="16384" width="10.796875" style="11"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:38">
@@ -39949,7 +39950,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="2" spans="1:38" ht="16.5">
+    <row r="2" spans="1:38" ht="16.8">
       <c r="A2" s="33" t="s">
         <v>263</v>
       </c>
@@ -40100,7 +40101,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="3" spans="1:38" ht="16.5">
+    <row r="3" spans="1:38" ht="16.8">
       <c r="A3" s="33" t="s">
         <v>264</v>
       </c>
@@ -40251,7 +40252,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="4" spans="1:38" ht="16.5">
+    <row r="4" spans="1:38" ht="16.8">
       <c r="A4" s="33" t="s">
         <v>265</v>
       </c>
@@ -40402,7 +40403,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="5" spans="1:38" ht="16.5">
+    <row r="5" spans="1:38" ht="16.8">
       <c r="A5" s="33" t="s">
         <v>266</v>
       </c>
@@ -40566,19 +40567,19 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{99E94645-B80F-0D4E-B109-C05D67A154E2}">
   <dimension ref="A1:AL7"/>
-  <sheetFormatPr defaultColWidth="10.83203125" defaultRowHeight="15.5"/>
+  <sheetFormatPr defaultColWidth="10.796875" defaultRowHeight="15.6"/>
   <cols>
-    <col min="1" max="1" width="106.33203125" style="11" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="17.33203125" style="11" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="23.33203125" style="11" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="106.296875" style="11" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.296875" style="11" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="23.296875" style="11" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="9" style="11" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="23.83203125" style="11" bestFit="1" customWidth="1"/>
-    <col min="6" max="10" width="10.83203125" style="11"/>
-    <col min="11" max="11" width="15.33203125" style="11" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="18.33203125" style="28" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="23.796875" style="11" bestFit="1" customWidth="1"/>
+    <col min="6" max="10" width="10.796875" style="11"/>
+    <col min="11" max="11" width="15.296875" style="11" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="18.296875" style="28" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="15" style="11" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="19.5" style="11" bestFit="1" customWidth="1"/>
-    <col min="15" max="16384" width="10.83203125" style="11"/>
+    <col min="15" max="16384" width="10.796875" style="11"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:38">
@@ -40697,7 +40698,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="2" spans="1:38" ht="16.5">
+    <row r="2" spans="1:38" ht="16.8">
       <c r="A2" s="32" t="s">
         <v>267</v>
       </c>
@@ -40848,7 +40849,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="3" spans="1:38" ht="16.5">
+    <row r="3" spans="1:38" ht="16.8">
       <c r="A3" s="32" t="s">
         <v>268</v>
       </c>
@@ -40999,7 +41000,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="4" spans="1:38" ht="16.5">
+    <row r="4" spans="1:38" ht="16.8">
       <c r="A4" s="32" t="s">
         <v>269</v>
       </c>
@@ -41150,7 +41151,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="5" spans="1:38" ht="16.5">
+    <row r="5" spans="1:38" ht="16.8">
       <c r="A5" s="32" t="s">
         <v>270</v>
       </c>
@@ -41301,7 +41302,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="6" spans="1:38" ht="16.5">
+    <row r="6" spans="1:38" ht="16.8">
       <c r="A6" s="32" t="s">
         <v>271</v>
       </c>
@@ -41452,7 +41453,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="7" spans="1:38" ht="16.5">
+    <row r="7" spans="1:38" ht="16.8">
       <c r="A7" s="32" t="s">
         <v>272</v>
       </c>
@@ -41745,18 +41746,18 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
   <Edit>DocumentLibraryForm</Edit>
   <New>DocumentLibraryForm</New>
 </FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -41778,14 +41779,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BD641CF5-135D-42FC-A55D-82791A85B476}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3C30B22D-1747-44FE-B15C-A00BE24DA1E1}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
@@ -41799,4 +41792,12 @@
     <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BD641CF5-135D-42FC-A55D-82791A85B476}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
updated shipment product in testcasesmapping
</commit_message>
<xml_diff>
--- a/CargoUIAutomationNew/src/test/resources/TestCasesMapping.xlsx
+++ b/CargoUIAutomationNew/src/test/resources/TestCasesMapping.xlsx
@@ -5,12 +5,12 @@
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\p57448\Desktop\Drafts\My Repo Excelbackup\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\p57448\Desktop\Cargo_B\Cargo\CargoUIAutomationNew\src\test\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{A29A29C6-B167-4455-BD00-2A3DF67FD2C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F88D73FF-7ED1-4686-9DBF-040B049153AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" firstSheet="1" activeTab="3" xr2:uid="{1AB005B2-AFEC-3B46-93EF-50FA3BE3C5FF}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" activeTab="2" xr2:uid="{1AB005B2-AFEC-3B46-93EF-50FA3BE3C5FF}"/>
   </bookViews>
   <sheets>
     <sheet name="Configuration" sheetId="14" r:id="rId1"/>
@@ -1099,27 +1099,6 @@
     <t>createAndConfirmGuidedBookingValuables_SAFE_Valuelessthan25000USD_International</t>
   </si>
   <si>
-    <t>CARE</t>
-  </si>
-  <si>
-    <t>createAndConfirmGuidedBookingHumanRemains_CARE_Adult_Domestic</t>
-  </si>
-  <si>
-    <t>createAndConfirmGuidedBookingHumanRemains_CARE_ChildInfant_Domestic</t>
-  </si>
-  <si>
-    <t>createAndConfirmGuidedBookingHumanRemains_CARE_CrematedRemains_Domestic</t>
-  </si>
-  <si>
-    <t>createAndConfirmGuidedBookingHumanRemains_CARE_Adult_International</t>
-  </si>
-  <si>
-    <t>createAndConfirmGuidedBookingHumanRemains_CARE_ChildInfant_International</t>
-  </si>
-  <si>
-    <t>createAndConfirmGuidedBookingHumanRemains_CARE_CrematedRemains_International</t>
-  </si>
-  <si>
     <t>createAndConfirmAdvanceBookingGeneral_Cargo_STANDARD_Loose_Domestic</t>
   </si>
   <si>
@@ -1304,6 +1283,27 @@
   </si>
   <si>
     <t>createAndConfirmAdvanceBookingLiveAnimals_LIVE_HatchingEggs_International</t>
+  </si>
+  <si>
+    <t>Cares</t>
+  </si>
+  <si>
+    <t>createAndConfirmGuidedBookingHumanRemains_Cares_Adult_Domestic</t>
+  </si>
+  <si>
+    <t>createAndConfirmGuidedBookingHumanRemains_Cares_ChildInfant_Domestic</t>
+  </si>
+  <si>
+    <t>createAndConfirmGuidedBookingHumanRemains_Cares_CrematedRemains_Domestic</t>
+  </si>
+  <si>
+    <t>createAndConfirmGuidedBookingHumanRemains_Cares_Adult_International</t>
+  </si>
+  <si>
+    <t>createAndConfirmGuidedBookingHumanRemains_Cares_ChildInfant_International</t>
+  </si>
+  <si>
+    <t>createAndConfirmGuidedBookingHumanRemains_Cares_CrematedRemains_International</t>
   </si>
 </sst>
 </file>
@@ -2367,7 +2367,7 @@
     </row>
     <row r="2" spans="1:38" ht="17" thickBot="1">
       <c r="A2" s="75" t="s">
-        <v>394</v>
+        <v>387</v>
       </c>
       <c r="B2" s="32" t="s">
         <v>210</v>
@@ -2518,7 +2518,7 @@
     </row>
     <row r="3" spans="1:38" ht="17" thickBot="1">
       <c r="A3" s="75" t="s">
-        <v>395</v>
+        <v>388</v>
       </c>
       <c r="B3" s="32" t="s">
         <v>210</v>
@@ -2669,7 +2669,7 @@
     </row>
     <row r="4" spans="1:38" ht="17" thickBot="1">
       <c r="A4" s="75" t="s">
-        <v>396</v>
+        <v>389</v>
       </c>
       <c r="B4" s="32" t="s">
         <v>210</v>
@@ -2820,7 +2820,7 @@
     </row>
     <row r="5" spans="1:38" ht="17" thickBot="1">
       <c r="A5" s="75" t="s">
-        <v>397</v>
+        <v>390</v>
       </c>
       <c r="B5" s="32" t="s">
         <v>210</v>
@@ -2971,7 +2971,7 @@
     </row>
     <row r="6" spans="1:38" ht="17" thickBot="1">
       <c r="A6" s="75" t="s">
-        <v>398</v>
+        <v>391</v>
       </c>
       <c r="B6" s="32" t="s">
         <v>210</v>
@@ -3122,7 +3122,7 @@
     </row>
     <row r="7" spans="1:38" ht="17" thickBot="1">
       <c r="A7" s="75" t="s">
-        <v>399</v>
+        <v>392</v>
       </c>
       <c r="B7" s="32" t="s">
         <v>210</v>
@@ -3273,7 +3273,7 @@
     </row>
     <row r="8" spans="1:38" ht="17" thickBot="1">
       <c r="A8" s="75" t="s">
-        <v>400</v>
+        <v>393</v>
       </c>
       <c r="B8" s="32" t="s">
         <v>210</v>
@@ -3424,7 +3424,7 @@
     </row>
     <row r="9" spans="1:38" ht="17" thickBot="1">
       <c r="A9" s="75" t="s">
-        <v>401</v>
+        <v>394</v>
       </c>
       <c r="B9" s="32" t="s">
         <v>210</v>
@@ -3575,7 +3575,7 @@
     </row>
     <row r="10" spans="1:38" ht="17" thickBot="1">
       <c r="A10" s="75" t="s">
-        <v>402</v>
+        <v>395</v>
       </c>
       <c r="B10" s="32" t="s">
         <v>210</v>
@@ -3726,7 +3726,7 @@
     </row>
     <row r="11" spans="1:38" ht="17" thickBot="1">
       <c r="A11" s="75" t="s">
-        <v>403</v>
+        <v>396</v>
       </c>
       <c r="B11" s="32" t="s">
         <v>210</v>
@@ -3877,7 +3877,7 @@
     </row>
     <row r="12" spans="1:38" ht="17" thickBot="1">
       <c r="A12" s="75" t="s">
-        <v>404</v>
+        <v>397</v>
       </c>
       <c r="B12" s="32" t="s">
         <v>210</v>
@@ -4028,7 +4028,7 @@
     </row>
     <row r="13" spans="1:38" ht="17" thickBot="1">
       <c r="A13" s="75" t="s">
-        <v>405</v>
+        <v>398</v>
       </c>
       <c r="B13" s="32" t="s">
         <v>210</v>
@@ -4179,7 +4179,7 @@
     </row>
     <row r="14" spans="1:38" ht="17" thickBot="1">
       <c r="A14" s="75" t="s">
-        <v>406</v>
+        <v>399</v>
       </c>
       <c r="B14" s="32" t="s">
         <v>210</v>
@@ -4330,7 +4330,7 @@
     </row>
     <row r="15" spans="1:38" ht="17" thickBot="1">
       <c r="A15" s="75" t="s">
-        <v>407</v>
+        <v>400</v>
       </c>
       <c r="B15" s="32" t="s">
         <v>210</v>
@@ -17519,13 +17519,13 @@
     </row>
     <row r="2" spans="1:39" ht="16" thickBot="1">
       <c r="A2" s="70" t="s">
-        <v>340</v>
+        <v>402</v>
       </c>
       <c r="B2" s="42" t="s">
         <v>311</v>
       </c>
       <c r="C2" s="11" t="s">
-        <v>339</v>
+        <v>401</v>
       </c>
       <c r="D2" s="40" t="str">
         <f>IF(TestCaseConfig!$B$2="Yes","Yes","No")</f>
@@ -17533,7 +17533,7 @@
       </c>
       <c r="E2" s="31" t="str" cm="1">
         <f t="array" ref="E2">_xlfn.XLOOKUP($A2,DataColumnRange,_xlfn.XLOOKUP(E$1,dataRowRange,ActualDataRange))</f>
-        <v>CARE</v>
+        <v>Cares</v>
       </c>
       <c r="F2" s="31" t="str" cm="1">
         <f t="array" ref="F2">_xlfn.XLOOKUP($A2,DataColumnRange,_xlfn.XLOOKUP(F$1,dataRowRange,ActualDataRange))</f>
@@ -17674,13 +17674,13 @@
     </row>
     <row r="3" spans="1:39" ht="16" thickBot="1">
       <c r="A3" s="71" t="s">
-        <v>341</v>
+        <v>403</v>
       </c>
       <c r="B3" s="42" t="s">
         <v>311</v>
       </c>
       <c r="C3" s="11" t="s">
-        <v>339</v>
+        <v>401</v>
       </c>
       <c r="D3" s="40" t="str">
         <f>IF(TestCaseConfig!$B$2="Yes","Yes","No")</f>
@@ -17688,7 +17688,7 @@
       </c>
       <c r="E3" s="31" t="str" cm="1">
         <f t="array" ref="E3">_xlfn.XLOOKUP($A3,DataColumnRange,_xlfn.XLOOKUP(E$1,dataRowRange,ActualDataRange))</f>
-        <v>CARE</v>
+        <v>Cares</v>
       </c>
       <c r="F3" s="31" t="str" cm="1">
         <f t="array" ref="F3">_xlfn.XLOOKUP($A3,DataColumnRange,_xlfn.XLOOKUP(F$1,dataRowRange,ActualDataRange))</f>
@@ -17829,13 +17829,13 @@
     </row>
     <row r="4" spans="1:39" ht="16" thickBot="1">
       <c r="A4" s="71" t="s">
-        <v>342</v>
+        <v>404</v>
       </c>
       <c r="B4" s="42" t="s">
         <v>311</v>
       </c>
       <c r="C4" s="11" t="s">
-        <v>339</v>
+        <v>401</v>
       </c>
       <c r="D4" s="40" t="str">
         <f>IF(TestCaseConfig!$B$2="Yes","Yes","No")</f>
@@ -17843,7 +17843,7 @@
       </c>
       <c r="E4" s="31" t="str" cm="1">
         <f t="array" ref="E4">_xlfn.XLOOKUP($A4,DataColumnRange,_xlfn.XLOOKUP(E$1,dataRowRange,ActualDataRange))</f>
-        <v>CARE</v>
+        <v>Cares</v>
       </c>
       <c r="F4" s="31" t="str" cm="1">
         <f t="array" ref="F4">_xlfn.XLOOKUP($A4,DataColumnRange,_xlfn.XLOOKUP(F$1,dataRowRange,ActualDataRange))</f>
@@ -17984,13 +17984,13 @@
     </row>
     <row r="5" spans="1:39" ht="16" thickBot="1">
       <c r="A5" s="71" t="s">
-        <v>343</v>
+        <v>405</v>
       </c>
       <c r="B5" s="42" t="s">
         <v>311</v>
       </c>
       <c r="C5" s="11" t="s">
-        <v>339</v>
+        <v>401</v>
       </c>
       <c r="D5" s="40" t="str">
         <f>IF(TestCaseConfig!$B$2="Yes","Yes","No")</f>
@@ -17998,7 +17998,7 @@
       </c>
       <c r="E5" s="31" t="str" cm="1">
         <f t="array" ref="E5">_xlfn.XLOOKUP($A5,DataColumnRange,_xlfn.XLOOKUP(E$1,dataRowRange,ActualDataRange))</f>
-        <v>CARE</v>
+        <v>Cares</v>
       </c>
       <c r="F5" s="31" t="str" cm="1">
         <f t="array" ref="F5">_xlfn.XLOOKUP($A5,DataColumnRange,_xlfn.XLOOKUP(F$1,dataRowRange,ActualDataRange))</f>
@@ -18139,13 +18139,13 @@
     </row>
     <row r="6" spans="1:39" ht="16" thickBot="1">
       <c r="A6" s="71" t="s">
-        <v>344</v>
+        <v>406</v>
       </c>
       <c r="B6" s="42" t="s">
         <v>311</v>
       </c>
       <c r="C6" s="11" t="s">
-        <v>339</v>
+        <v>401</v>
       </c>
       <c r="D6" s="40" t="str">
         <f>IF(TestCaseConfig!$B$2="Yes","Yes","No")</f>
@@ -18153,7 +18153,7 @@
       </c>
       <c r="E6" s="31" t="str" cm="1">
         <f t="array" ref="E6">_xlfn.XLOOKUP($A6,DataColumnRange,_xlfn.XLOOKUP(E$1,dataRowRange,ActualDataRange))</f>
-        <v>CARE</v>
+        <v>Cares</v>
       </c>
       <c r="F6" s="31" t="str" cm="1">
         <f t="array" ref="F6">_xlfn.XLOOKUP($A6,DataColumnRange,_xlfn.XLOOKUP(F$1,dataRowRange,ActualDataRange))</f>
@@ -18294,13 +18294,13 @@
     </row>
     <row r="7" spans="1:39" ht="16" thickBot="1">
       <c r="A7" s="71" t="s">
-        <v>345</v>
+        <v>407</v>
       </c>
       <c r="B7" s="42" t="s">
         <v>311</v>
       </c>
       <c r="C7" s="11" t="s">
-        <v>339</v>
+        <v>401</v>
       </c>
       <c r="D7" s="40" t="str">
         <f>IF(TestCaseConfig!$B$2="Yes","Yes","No")</f>
@@ -18308,7 +18308,7 @@
       </c>
       <c r="E7" s="31" t="str" cm="1">
         <f t="array" ref="E7">_xlfn.XLOOKUP($A7,DataColumnRange,_xlfn.XLOOKUP(E$1,dataRowRange,ActualDataRange))</f>
-        <v>CARE</v>
+        <v>Cares</v>
       </c>
       <c r="F7" s="31" t="str" cm="1">
         <f t="array" ref="F7">_xlfn.XLOOKUP($A7,DataColumnRange,_xlfn.XLOOKUP(F$1,dataRowRange,ActualDataRange))</f>
@@ -32565,13 +32565,13 @@
     <row r="124" spans="1:36" s="61" customFormat="1">
       <c r="A124" s="61" t="str">
         <f t="shared" si="1"/>
-        <v>createAndConfirmGuidedBookingHumanRemains_CARE_Adult_Domestic</v>
+        <v>createAndConfirmGuidedBookingHumanRemains_Cares_Adult_Domestic</v>
       </c>
       <c r="B124" s="61" t="s">
         <v>311</v>
       </c>
       <c r="C124" s="61" t="s">
-        <v>339</v>
+        <v>401</v>
       </c>
       <c r="D124" s="46" t="s">
         <v>125</v>
@@ -32676,13 +32676,13 @@
     <row r="125" spans="1:36" s="61" customFormat="1">
       <c r="A125" s="61" t="str">
         <f t="shared" si="1"/>
-        <v>createAndConfirmGuidedBookingHumanRemains_CARE_ChildInfant_Domestic</v>
+        <v>createAndConfirmGuidedBookingHumanRemains_Cares_ChildInfant_Domestic</v>
       </c>
       <c r="B125" s="61" t="s">
         <v>311</v>
       </c>
       <c r="C125" s="61" t="s">
-        <v>339</v>
+        <v>401</v>
       </c>
       <c r="D125" s="46" t="s">
         <v>125</v>
@@ -32787,13 +32787,13 @@
     <row r="126" spans="1:36" s="61" customFormat="1">
       <c r="A126" s="61" t="str">
         <f t="shared" si="1"/>
-        <v>createAndConfirmGuidedBookingHumanRemains_CARE_CrematedRemains_Domestic</v>
+        <v>createAndConfirmGuidedBookingHumanRemains_Cares_CrematedRemains_Domestic</v>
       </c>
       <c r="B126" s="61" t="s">
         <v>311</v>
       </c>
       <c r="C126" s="61" t="s">
-        <v>339</v>
+        <v>401</v>
       </c>
       <c r="D126" s="46" t="s">
         <v>125</v>
@@ -32898,13 +32898,13 @@
     <row r="127" spans="1:36" s="61" customFormat="1">
       <c r="A127" s="61" t="str">
         <f t="shared" si="1"/>
-        <v>createAndConfirmGuidedBookingHumanRemains_CARE_Adult_International</v>
+        <v>createAndConfirmGuidedBookingHumanRemains_Cares_Adult_International</v>
       </c>
       <c r="B127" s="61" t="s">
         <v>311</v>
       </c>
       <c r="C127" s="61" t="s">
-        <v>339</v>
+        <v>401</v>
       </c>
       <c r="D127" s="46" t="s">
         <v>125</v>
@@ -33009,13 +33009,13 @@
     <row r="128" spans="1:36" s="61" customFormat="1">
       <c r="A128" s="61" t="str">
         <f t="shared" si="1"/>
-        <v>createAndConfirmGuidedBookingHumanRemains_CARE_ChildInfant_International</v>
+        <v>createAndConfirmGuidedBookingHumanRemains_Cares_ChildInfant_International</v>
       </c>
       <c r="B128" s="61" t="s">
         <v>311</v>
       </c>
       <c r="C128" s="61" t="s">
-        <v>339</v>
+        <v>401</v>
       </c>
       <c r="D128" s="46" t="s">
         <v>125</v>
@@ -33120,13 +33120,13 @@
     <row r="129" spans="1:36" s="61" customFormat="1">
       <c r="A129" s="61" t="str">
         <f t="shared" ref="A129" si="2">_xlfn.CONCAT("createAndConfirmGuidedBooking",SUBSTITUTE(B129," ","_"),"_",SUBSTITUTE(C129," ","_"),"_",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(J129," ",""),"-",""),"/",""),"–",""),"+",""),"°",""),",",""),"_",SUBSTITUTE(AJ129," ","_"))</f>
-        <v>createAndConfirmGuidedBookingHumanRemains_CARE_CrematedRemains_International</v>
+        <v>createAndConfirmGuidedBookingHumanRemains_Cares_CrematedRemains_International</v>
       </c>
       <c r="B129" s="61" t="s">
         <v>311</v>
       </c>
       <c r="C129" s="61" t="s">
-        <v>339</v>
+        <v>401</v>
       </c>
       <c r="D129" s="46" t="s">
         <v>125</v>
@@ -33537,7 +33537,7 @@
     </row>
     <row r="2" spans="1:41" ht="16.5" thickBot="1">
       <c r="A2" s="74" t="s">
-        <v>346</v>
+        <v>339</v>
       </c>
       <c r="B2" s="38" t="str" cm="1">
         <f t="array" ref="B2">_xlfn.XLOOKUP($A2,DataColumnRange,_xlfn.XLOOKUP(B$1,dataRowRange,ActualDataRange))</f>
@@ -33700,7 +33700,7 @@
     </row>
     <row r="3" spans="1:41" ht="16.5" thickBot="1">
       <c r="A3" s="75" t="s">
-        <v>347</v>
+        <v>340</v>
       </c>
       <c r="B3" s="38" t="str" cm="1">
         <f t="array" ref="B3">_xlfn.XLOOKUP($A3,DataColumnRange,_xlfn.XLOOKUP(B$1,dataRowRange,ActualDataRange))</f>
@@ -33863,7 +33863,7 @@
     </row>
     <row r="4" spans="1:41" ht="16.5" thickBot="1">
       <c r="A4" s="75" t="s">
-        <v>348</v>
+        <v>341</v>
       </c>
       <c r="B4" s="38" t="str" cm="1">
         <f t="array" ref="B4">_xlfn.XLOOKUP($A4,DataColumnRange,_xlfn.XLOOKUP(B$1,dataRowRange,ActualDataRange))</f>
@@ -34027,7 +34027,7 @@
     </row>
     <row r="5" spans="1:41" ht="16.5" thickBot="1">
       <c r="A5" s="75" t="s">
-        <v>349</v>
+        <v>342</v>
       </c>
       <c r="B5" s="38" t="str" cm="1">
         <f t="array" ref="B5">_xlfn.XLOOKUP($A5,DataColumnRange,_xlfn.XLOOKUP(B$1,dataRowRange,ActualDataRange))</f>
@@ -34191,7 +34191,7 @@
     </row>
     <row r="6" spans="1:41" ht="16.5" thickBot="1">
       <c r="A6" s="75" t="s">
-        <v>350</v>
+        <v>343</v>
       </c>
       <c r="B6" s="38" t="str" cm="1">
         <f t="array" ref="B6">_xlfn.XLOOKUP($A6,DataColumnRange,_xlfn.XLOOKUP(B$1,dataRowRange,ActualDataRange))</f>
@@ -34355,7 +34355,7 @@
     </row>
     <row r="7" spans="1:41" ht="16.5" thickBot="1">
       <c r="A7" s="75" t="s">
-        <v>351</v>
+        <v>344</v>
       </c>
       <c r="B7" s="38" t="str" cm="1">
         <f t="array" ref="B7">_xlfn.XLOOKUP($A7,DataColumnRange,_xlfn.XLOOKUP(B$1,dataRowRange,ActualDataRange))</f>
@@ -34687,7 +34687,7 @@
     </row>
     <row r="2" spans="1:38" ht="17" thickBot="1">
       <c r="A2" s="75" t="s">
-        <v>352</v>
+        <v>345</v>
       </c>
       <c r="B2" s="33" t="s">
         <v>47</v>
@@ -34838,7 +34838,7 @@
     </row>
     <row r="3" spans="1:38" ht="17" thickBot="1">
       <c r="A3" s="75" t="s">
-        <v>353</v>
+        <v>346</v>
       </c>
       <c r="B3" s="33" t="s">
         <v>47</v>
@@ -34989,7 +34989,7 @@
     </row>
     <row r="4" spans="1:38" ht="17" thickBot="1">
       <c r="A4" s="75" t="s">
-        <v>354</v>
+        <v>347</v>
       </c>
       <c r="B4" s="33" t="s">
         <v>47</v>
@@ -35140,7 +35140,7 @@
     </row>
     <row r="5" spans="1:38" ht="17" thickBot="1">
       <c r="A5" s="75" t="s">
-        <v>355</v>
+        <v>348</v>
       </c>
       <c r="B5" s="33" t="s">
         <v>47</v>
@@ -35291,7 +35291,7 @@
     </row>
     <row r="6" spans="1:38" ht="17" thickBot="1">
       <c r="A6" s="75" t="s">
-        <v>356</v>
+        <v>349</v>
       </c>
       <c r="B6" s="33" t="s">
         <v>47</v>
@@ -35442,7 +35442,7 @@
     </row>
     <row r="7" spans="1:38" ht="17" thickBot="1">
       <c r="A7" s="75" t="s">
-        <v>357</v>
+        <v>350</v>
       </c>
       <c r="B7" s="33" t="s">
         <v>47</v>
@@ -35593,7 +35593,7 @@
     </row>
     <row r="8" spans="1:38" ht="17" thickBot="1">
       <c r="A8" s="75" t="s">
-        <v>358</v>
+        <v>351</v>
       </c>
       <c r="B8" s="33" t="s">
         <v>47</v>
@@ -35744,7 +35744,7 @@
     </row>
     <row r="9" spans="1:38" ht="17" thickBot="1">
       <c r="A9" s="75" t="s">
-        <v>359</v>
+        <v>352</v>
       </c>
       <c r="B9" s="33" t="s">
         <v>47</v>
@@ -35895,7 +35895,7 @@
     </row>
     <row r="10" spans="1:38" ht="17" thickBot="1">
       <c r="A10" s="75" t="s">
-        <v>360</v>
+        <v>353</v>
       </c>
       <c r="B10" s="33" t="s">
         <v>47</v>
@@ -36046,7 +36046,7 @@
     </row>
     <row r="11" spans="1:38" ht="17" thickBot="1">
       <c r="A11" s="75" t="s">
-        <v>361</v>
+        <v>354</v>
       </c>
       <c r="B11" s="33" t="s">
         <v>47</v>
@@ -36341,7 +36341,7 @@
     </row>
     <row r="2" spans="1:38" ht="17" thickBot="1">
       <c r="A2" s="75" t="s">
-        <v>362</v>
+        <v>355</v>
       </c>
       <c r="B2" s="33" t="s">
         <v>58</v>
@@ -36492,7 +36492,7 @@
     </row>
     <row r="3" spans="1:38" ht="17" thickBot="1">
       <c r="A3" s="75" t="s">
-        <v>363</v>
+        <v>356</v>
       </c>
       <c r="B3" s="33" t="s">
         <v>58</v>
@@ -36643,7 +36643,7 @@
     </row>
     <row r="4" spans="1:38" ht="17" thickBot="1">
       <c r="A4" s="75" t="s">
-        <v>364</v>
+        <v>357</v>
       </c>
       <c r="B4" s="33" t="s">
         <v>58</v>
@@ -36794,7 +36794,7 @@
     </row>
     <row r="5" spans="1:38" ht="17" thickBot="1">
       <c r="A5" s="75" t="s">
-        <v>365</v>
+        <v>358</v>
       </c>
       <c r="B5" s="33" t="s">
         <v>58</v>
@@ -36945,7 +36945,7 @@
     </row>
     <row r="6" spans="1:38" ht="17" thickBot="1">
       <c r="A6" s="75" t="s">
-        <v>366</v>
+        <v>359</v>
       </c>
       <c r="B6" s="33" t="s">
         <v>58</v>
@@ -37096,7 +37096,7 @@
     </row>
     <row r="7" spans="1:38" ht="17" thickBot="1">
       <c r="A7" s="75" t="s">
-        <v>367</v>
+        <v>360</v>
       </c>
       <c r="B7" s="33" t="s">
         <v>58</v>
@@ -37247,7 +37247,7 @@
     </row>
     <row r="8" spans="1:38" ht="17" thickBot="1">
       <c r="A8" s="75" t="s">
-        <v>368</v>
+        <v>361</v>
       </c>
       <c r="B8" s="33" t="s">
         <v>58</v>
@@ -37398,7 +37398,7 @@
     </row>
     <row r="9" spans="1:38" ht="17" thickBot="1">
       <c r="A9" s="75" t="s">
-        <v>369</v>
+        <v>362</v>
       </c>
       <c r="B9" s="33" t="s">
         <v>58</v>
@@ -37549,7 +37549,7 @@
     </row>
     <row r="10" spans="1:38" ht="17" thickBot="1">
       <c r="A10" s="75" t="s">
-        <v>370</v>
+        <v>363</v>
       </c>
       <c r="B10" s="33" t="s">
         <v>58</v>
@@ -37700,7 +37700,7 @@
     </row>
     <row r="11" spans="1:38" ht="17" thickBot="1">
       <c r="A11" s="75" t="s">
-        <v>371</v>
+        <v>364</v>
       </c>
       <c r="B11" s="33" t="s">
         <v>58</v>
@@ -37993,7 +37993,7 @@
     </row>
     <row r="2" spans="1:38" ht="17" thickBot="1">
       <c r="A2" s="75" t="s">
-        <v>372</v>
+        <v>365</v>
       </c>
       <c r="B2" s="32" t="s">
         <v>44</v>
@@ -38144,7 +38144,7 @@
     </row>
     <row r="3" spans="1:38" ht="17" thickBot="1">
       <c r="A3" s="75" t="s">
-        <v>373</v>
+        <v>366</v>
       </c>
       <c r="B3" s="32" t="s">
         <v>44</v>
@@ -38295,7 +38295,7 @@
     </row>
     <row r="4" spans="1:38" ht="17" thickBot="1">
       <c r="A4" s="75" t="s">
-        <v>374</v>
+        <v>367</v>
       </c>
       <c r="B4" s="32" t="s">
         <v>44</v>
@@ -38446,7 +38446,7 @@
     </row>
     <row r="5" spans="1:38" ht="17" thickBot="1">
       <c r="A5" s="75" t="s">
-        <v>375</v>
+        <v>368</v>
       </c>
       <c r="B5" s="32" t="s">
         <v>44</v>
@@ -38597,7 +38597,7 @@
     </row>
     <row r="6" spans="1:38" ht="17" thickBot="1">
       <c r="A6" s="75" t="s">
-        <v>376</v>
+        <v>369</v>
       </c>
       <c r="B6" s="32" t="s">
         <v>44</v>
@@ -38748,7 +38748,7 @@
     </row>
     <row r="7" spans="1:38" ht="17" thickBot="1">
       <c r="A7" s="75" t="s">
-        <v>377</v>
+        <v>370</v>
       </c>
       <c r="B7" s="32" t="s">
         <v>44</v>
@@ -38899,7 +38899,7 @@
     </row>
     <row r="8" spans="1:38" ht="17" thickBot="1">
       <c r="A8" s="75" t="s">
-        <v>378</v>
+        <v>371</v>
       </c>
       <c r="B8" s="32" t="s">
         <v>44</v>
@@ -39050,7 +39050,7 @@
     </row>
     <row r="9" spans="1:38" ht="17" thickBot="1">
       <c r="A9" s="75" t="s">
-        <v>379</v>
+        <v>372</v>
       </c>
       <c r="B9" s="32" t="s">
         <v>44</v>
@@ -39201,7 +39201,7 @@
     </row>
     <row r="10" spans="1:38" ht="17" thickBot="1">
       <c r="A10" s="75" t="s">
-        <v>380</v>
+        <v>373</v>
       </c>
       <c r="B10" s="32" t="s">
         <v>44</v>
@@ -39352,7 +39352,7 @@
     </row>
     <row r="11" spans="1:38" ht="17" thickBot="1">
       <c r="A11" s="75" t="s">
-        <v>381</v>
+        <v>374</v>
       </c>
       <c r="B11" s="32" t="s">
         <v>44</v>
@@ -39503,7 +39503,7 @@
     </row>
     <row r="12" spans="1:38" ht="17" thickBot="1">
       <c r="A12" s="75" t="s">
-        <v>382</v>
+        <v>375</v>
       </c>
       <c r="B12" s="32" t="s">
         <v>44</v>
@@ -39654,7 +39654,7 @@
     </row>
     <row r="13" spans="1:38" ht="17" thickBot="1">
       <c r="A13" s="75" t="s">
-        <v>383</v>
+        <v>376</v>
       </c>
       <c r="B13" s="32" t="s">
         <v>44</v>
@@ -39948,7 +39948,7 @@
     </row>
     <row r="2" spans="1:38" ht="17" thickBot="1">
       <c r="A2" s="75" t="s">
-        <v>384</v>
+        <v>377</v>
       </c>
       <c r="B2" s="33" t="s">
         <v>87</v>
@@ -40099,7 +40099,7 @@
     </row>
     <row r="3" spans="1:38" ht="17" thickBot="1">
       <c r="A3" s="75" t="s">
-        <v>385</v>
+        <v>378</v>
       </c>
       <c r="B3" s="33" t="s">
         <v>87</v>
@@ -40250,7 +40250,7 @@
     </row>
     <row r="4" spans="1:38" ht="17" thickBot="1">
       <c r="A4" s="75" t="s">
-        <v>386</v>
+        <v>379</v>
       </c>
       <c r="B4" s="33" t="s">
         <v>87</v>
@@ -40401,7 +40401,7 @@
     </row>
     <row r="5" spans="1:38" ht="17" thickBot="1">
       <c r="A5" s="75" t="s">
-        <v>387</v>
+        <v>380</v>
       </c>
       <c r="B5" s="33" t="s">
         <v>87</v>
@@ -40696,7 +40696,7 @@
     </row>
     <row r="2" spans="1:38" ht="17" thickBot="1">
       <c r="A2" s="75" t="s">
-        <v>388</v>
+        <v>381</v>
       </c>
       <c r="B2" s="32" t="s">
         <v>89</v>
@@ -40847,7 +40847,7 @@
     </row>
     <row r="3" spans="1:38" ht="17" thickBot="1">
       <c r="A3" s="75" t="s">
-        <v>389</v>
+        <v>382</v>
       </c>
       <c r="B3" s="32" t="s">
         <v>89</v>
@@ -40998,7 +40998,7 @@
     </row>
     <row r="4" spans="1:38" ht="17" thickBot="1">
       <c r="A4" s="75" t="s">
-        <v>390</v>
+        <v>383</v>
       </c>
       <c r="B4" s="32" t="s">
         <v>89</v>
@@ -41149,7 +41149,7 @@
     </row>
     <row r="5" spans="1:38" ht="17" thickBot="1">
       <c r="A5" s="75" t="s">
-        <v>391</v>
+        <v>384</v>
       </c>
       <c r="B5" s="32" t="s">
         <v>89</v>
@@ -41300,7 +41300,7 @@
     </row>
     <row r="6" spans="1:38" ht="17" thickBot="1">
       <c r="A6" s="75" t="s">
-        <v>392</v>
+        <v>385</v>
       </c>
       <c r="B6" s="32" t="s">
         <v>89</v>
@@ -41451,7 +41451,7 @@
     </row>
     <row r="7" spans="1:38" ht="17" thickBot="1">
       <c r="A7" s="75" t="s">
-        <v>393</v>
+        <v>386</v>
       </c>
       <c r="B7" s="32" t="s">
         <v>89</v>
@@ -41610,6 +41610,21 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100DFBCF867C5410147BDDAF2BCA37BA4E7" ma:contentTypeVersion="2" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="e24a40d5ebdbb3b92553f235188d50f6">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="2981db02-ca81-468a-9abd-70e82312b342" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="db49c26ce236f576151feb411775a695" ns2:_="">
     <xsd:import namespace="2981db02-ca81-468a-9abd-70e82312b342"/>
@@ -41741,22 +41756,31 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3C30B22D-1747-44FE-B15C-A00BE24DA1E1}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="2981db02-ca81-468a-9abd-70e82312b342"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BD641CF5-135D-42FC-A55D-82791A85B476}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EED3BB4E-382D-479A-B77C-6CB5E1CFD30D}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -41772,28 +41796,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BD641CF5-135D-42FC-A55D-82791A85B476}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3C30B22D-1747-44FE-B15C-A00BE24DA1E1}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="2981db02-ca81-468a-9abd-70e82312b342"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
updated age to 35 for child
</commit_message>
<xml_diff>
--- a/CargoUIAutomationNew/src/test/resources/TestCasesMapping.xlsx
+++ b/CargoUIAutomationNew/src/test/resources/TestCasesMapping.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\p57448\Desktop\Cargo_B\Cargo\CargoUIAutomationNew\src\test\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F88D73FF-7ED1-4686-9DBF-040B049153AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B728B9E9-3CDF-4A88-969B-5C6C1DFDCA7F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" activeTab="2" xr2:uid="{1AB005B2-AFEC-3B46-93EF-50FA3BE3C5FF}"/>
   </bookViews>
@@ -17724,7 +17724,7 @@
       </c>
       <c r="N3" s="31" cm="1">
         <f t="array" ref="N3">_xlfn.XLOOKUP($A3,DataColumnRange,_xlfn.XLOOKUP(N$1,dataRowRange,ActualDataRange))</f>
-        <v>49</v>
+        <v>35</v>
       </c>
       <c r="O3" s="31" t="str" cm="1">
         <f t="array" ref="O3">_xlfn.XLOOKUP($A3,DataColumnRange,_xlfn.XLOOKUP(O$1,dataRowRange,ActualDataRange))</f>
@@ -18189,7 +18189,7 @@
       </c>
       <c r="N6" s="31" cm="1">
         <f t="array" ref="N6">_xlfn.XLOOKUP($A6,DataColumnRange,_xlfn.XLOOKUP(N$1,dataRowRange,ActualDataRange))</f>
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="O6" s="31" t="str" cm="1">
         <f t="array" ref="O6">_xlfn.XLOOKUP($A6,DataColumnRange,_xlfn.XLOOKUP(O$1,dataRowRange,ActualDataRange))</f>
@@ -32709,7 +32709,7 @@
         <v>308</v>
       </c>
       <c r="L125" s="61">
-        <v>49</v>
+        <v>35</v>
       </c>
       <c r="M125" s="61" t="s">
         <v>145</v>
@@ -33042,7 +33042,7 @@
         <v>308</v>
       </c>
       <c r="L128" s="61">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="M128" s="61" t="s">
         <v>198</v>
@@ -41610,21 +41610,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100DFBCF867C5410147BDDAF2BCA37BA4E7" ma:contentTypeVersion="2" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="e24a40d5ebdbb3b92553f235188d50f6">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="2981db02-ca81-468a-9abd-70e82312b342" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="db49c26ce236f576151feb411775a695" ns2:_="">
     <xsd:import namespace="2981db02-ca81-468a-9abd-70e82312b342"/>
@@ -41756,31 +41741,22 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3C30B22D-1747-44FE-B15C-A00BE24DA1E1}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="2981db02-ca81-468a-9abd-70e82312b342"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BD641CF5-135D-42FC-A55D-82791A85B476}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EED3BB4E-382D-479A-B77C-6CB5E1CFD30D}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -41796,4 +41772,28 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BD641CF5-135D-42FC-A55D-82791A85B476}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3C30B22D-1747-44FE-B15C-A00BE24DA1E1}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="2981db02-ca81-468a-9abd-70e82312b342"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
updated CARE to Cares
</commit_message>
<xml_diff>
--- a/CargoUIAutomationNew/src/test/resources/TestCasesMapping.xlsx
+++ b/CargoUIAutomationNew/src/test/resources/TestCasesMapping.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\p57448\Desktop\Cargo_B\Cargo\CargoUIAutomationNew\src\test\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{130465E4-222D-4F23-AF9F-5549C932BCA9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C3A8BE43-9413-4083-9B71-24B7B62F9BCE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" firstSheet="1" activeTab="2" xr2:uid="{1AB005B2-AFEC-3B46-93EF-50FA3BE3C5FF}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" firstSheet="13" activeTab="18" xr2:uid="{1AB005B2-AFEC-3B46-93EF-50FA3BE3C5FF}"/>
   </bookViews>
   <sheets>
     <sheet name="Configuration" sheetId="14" r:id="rId1"/>
@@ -1096,27 +1096,6 @@
     <t>createAndConfirmGuidedBookingValuables_SAFE_Valuelessthan25000USD_International</t>
   </si>
   <si>
-    <t>CARE</t>
-  </si>
-  <si>
-    <t>createAndConfirmGuidedBookingHumanRemains_CARE_Adult_Domestic</t>
-  </si>
-  <si>
-    <t>createAndConfirmGuidedBookingHumanRemains_CARE_ChildInfant_Domestic</t>
-  </si>
-  <si>
-    <t>createAndConfirmGuidedBookingHumanRemains_CARE_CrematedRemains_Domestic</t>
-  </si>
-  <si>
-    <t>createAndConfirmGuidedBookingHumanRemains_CARE_Adult_International</t>
-  </si>
-  <si>
-    <t>createAndConfirmGuidedBookingHumanRemains_CARE_ChildInfant_International</t>
-  </si>
-  <si>
-    <t>createAndConfirmGuidedBookingHumanRemains_CARE_CrematedRemains_International</t>
-  </si>
-  <si>
     <t>createAndConfirmAdvanceBookingGeneral_Cargo_STANDARD_Loose_Domestic</t>
   </si>
   <si>
@@ -1308,14 +1287,42 @@
   <si>
     <t>Test Human Remains</t>
   </si>
+  <si>
+    <t>Cares</t>
+  </si>
+  <si>
+    <t>createAndConfirmGuidedBookingHumanRemains_Cares_Adult_Domestic</t>
+  </si>
+  <si>
+    <t>createAndConfirmGuidedBookingHumanRemains_Cares_ChildInfant_Domestic</t>
+  </si>
+  <si>
+    <t>createAndConfirmGuidedBookingHumanRemains_Cares_CrematedRemains_Domestic</t>
+  </si>
+  <si>
+    <t>createAndConfirmGuidedBookingHumanRemains_Cares_Adult_International</t>
+  </si>
+  <si>
+    <t>createAndConfirmGuidedBookingHumanRemains_Cares_ChildInfant_International</t>
+  </si>
+  <si>
+    <t>createAndConfirmGuidedBookingHumanRemains_Cares_CrematedRemains_International</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="10">
+  <fonts count="11">
     <font>
       <sz val="12"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -1635,9 +1642,9 @@
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="76">
+  <cellXfs count="77">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
@@ -1645,25 +1652,25 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
@@ -1671,25 +1678,25 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" quotePrefix="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="2" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="2" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="9" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1699,14 +1706,14 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1715,45 +1722,45 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="9" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="9" fillId="4" borderId="1" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="10" fillId="4" borderId="1" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1762,7 +1769,7 @@
     <xf numFmtId="49" fontId="0" fillId="4" borderId="1" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" quotePrefix="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1813,21 +1820,21 @@
     <xf numFmtId="0" fontId="0" fillId="14" borderId="1" xfId="0" quotePrefix="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="17" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="18" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="19" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="20" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="21" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="22" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="17" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="18" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="19" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="20" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="21" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="22" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="22" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="22" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="23" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="23" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="23" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="23" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1836,11 +1843,14 @@
     <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" quotePrefix="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -2370,7 +2380,7 @@
     </row>
     <row r="2" spans="1:38" ht="17" thickBot="1">
       <c r="A2" s="75" t="s">
-        <v>393</v>
+        <v>386</v>
       </c>
       <c r="B2" s="32" t="s">
         <v>209</v>
@@ -2521,7 +2531,7 @@
     </row>
     <row r="3" spans="1:38" ht="17" thickBot="1">
       <c r="A3" s="75" t="s">
-        <v>394</v>
+        <v>387</v>
       </c>
       <c r="B3" s="32" t="s">
         <v>209</v>
@@ -2672,7 +2682,7 @@
     </row>
     <row r="4" spans="1:38" ht="17" thickBot="1">
       <c r="A4" s="75" t="s">
-        <v>395</v>
+        <v>388</v>
       </c>
       <c r="B4" s="32" t="s">
         <v>209</v>
@@ -2823,7 +2833,7 @@
     </row>
     <row r="5" spans="1:38" ht="17" thickBot="1">
       <c r="A5" s="75" t="s">
-        <v>396</v>
+        <v>389</v>
       </c>
       <c r="B5" s="32" t="s">
         <v>209</v>
@@ -2974,7 +2984,7 @@
     </row>
     <row r="6" spans="1:38" ht="17" thickBot="1">
       <c r="A6" s="75" t="s">
-        <v>397</v>
+        <v>390</v>
       </c>
       <c r="B6" s="32" t="s">
         <v>209</v>
@@ -3125,7 +3135,7 @@
     </row>
     <row r="7" spans="1:38" ht="17" thickBot="1">
       <c r="A7" s="75" t="s">
-        <v>398</v>
+        <v>391</v>
       </c>
       <c r="B7" s="32" t="s">
         <v>209</v>
@@ -3276,7 +3286,7 @@
     </row>
     <row r="8" spans="1:38" ht="17" thickBot="1">
       <c r="A8" s="75" t="s">
-        <v>399</v>
+        <v>392</v>
       </c>
       <c r="B8" s="32" t="s">
         <v>209</v>
@@ -3427,7 +3437,7 @@
     </row>
     <row r="9" spans="1:38" ht="17" thickBot="1">
       <c r="A9" s="75" t="s">
-        <v>400</v>
+        <v>393</v>
       </c>
       <c r="B9" s="32" t="s">
         <v>209</v>
@@ -3578,7 +3588,7 @@
     </row>
     <row r="10" spans="1:38" ht="17" thickBot="1">
       <c r="A10" s="75" t="s">
-        <v>401</v>
+        <v>394</v>
       </c>
       <c r="B10" s="32" t="s">
         <v>209</v>
@@ -3729,7 +3739,7 @@
     </row>
     <row r="11" spans="1:38" ht="17" thickBot="1">
       <c r="A11" s="75" t="s">
-        <v>402</v>
+        <v>395</v>
       </c>
       <c r="B11" s="32" t="s">
         <v>209</v>
@@ -3880,7 +3890,7 @@
     </row>
     <row r="12" spans="1:38" ht="17" thickBot="1">
       <c r="A12" s="75" t="s">
-        <v>403</v>
+        <v>396</v>
       </c>
       <c r="B12" s="32" t="s">
         <v>209</v>
@@ -4031,7 +4041,7 @@
     </row>
     <row r="13" spans="1:38" ht="17" thickBot="1">
       <c r="A13" s="75" t="s">
-        <v>404</v>
+        <v>397</v>
       </c>
       <c r="B13" s="32" t="s">
         <v>209</v>
@@ -4182,7 +4192,7 @@
     </row>
     <row r="14" spans="1:38" ht="17" thickBot="1">
       <c r="A14" s="75" t="s">
-        <v>405</v>
+        <v>398</v>
       </c>
       <c r="B14" s="32" t="s">
         <v>209</v>
@@ -4333,7 +4343,7 @@
     </row>
     <row r="15" spans="1:38" ht="17" thickBot="1">
       <c r="A15" s="75" t="s">
-        <v>406</v>
+        <v>399</v>
       </c>
       <c r="B15" s="32" t="s">
         <v>209</v>
@@ -17522,13 +17532,13 @@
     </row>
     <row r="2" spans="1:39" ht="16" thickBot="1">
       <c r="A2" s="70" t="s">
-        <v>339</v>
+        <v>403</v>
       </c>
       <c r="B2" s="42" t="s">
         <v>310</v>
       </c>
       <c r="C2" s="11" t="s">
-        <v>338</v>
+        <v>402</v>
       </c>
       <c r="D2" s="40" t="str">
         <f>IF(TestCaseConfig!$B$2="Yes","Yes","No")</f>
@@ -17536,7 +17546,7 @@
       </c>
       <c r="E2" s="31" t="str" cm="1">
         <f t="array" ref="E2">_xlfn.XLOOKUP($A2,DataColumnRange,_xlfn.XLOOKUP(E$1,dataRowRange,ActualDataRange))</f>
-        <v>CARE</v>
+        <v>Cares</v>
       </c>
       <c r="F2" s="31" t="str" cm="1">
         <f t="array" ref="F2">_xlfn.XLOOKUP($A2,DataColumnRange,_xlfn.XLOOKUP(F$1,dataRowRange,ActualDataRange))</f>
@@ -17677,13 +17687,13 @@
     </row>
     <row r="3" spans="1:39" ht="16" thickBot="1">
       <c r="A3" s="71" t="s">
-        <v>340</v>
+        <v>404</v>
       </c>
       <c r="B3" s="42" t="s">
         <v>310</v>
       </c>
       <c r="C3" s="11" t="s">
-        <v>338</v>
+        <v>402</v>
       </c>
       <c r="D3" s="40" t="str">
         <f>IF(TestCaseConfig!$B$2="Yes","Yes","No")</f>
@@ -17691,7 +17701,7 @@
       </c>
       <c r="E3" s="31" t="str" cm="1">
         <f t="array" ref="E3">_xlfn.XLOOKUP($A3,DataColumnRange,_xlfn.XLOOKUP(E$1,dataRowRange,ActualDataRange))</f>
-        <v>CARE</v>
+        <v>Cares</v>
       </c>
       <c r="F3" s="31" t="str" cm="1">
         <f t="array" ref="F3">_xlfn.XLOOKUP($A3,DataColumnRange,_xlfn.XLOOKUP(F$1,dataRowRange,ActualDataRange))</f>
@@ -17832,13 +17842,13 @@
     </row>
     <row r="4" spans="1:39" ht="16" thickBot="1">
       <c r="A4" s="71" t="s">
-        <v>341</v>
+        <v>405</v>
       </c>
       <c r="B4" s="42" t="s">
         <v>310</v>
       </c>
       <c r="C4" s="11" t="s">
-        <v>338</v>
+        <v>402</v>
       </c>
       <c r="D4" s="40" t="str">
         <f>IF(TestCaseConfig!$B$2="Yes","Yes","No")</f>
@@ -17846,7 +17856,7 @@
       </c>
       <c r="E4" s="31" t="str" cm="1">
         <f t="array" ref="E4">_xlfn.XLOOKUP($A4,DataColumnRange,_xlfn.XLOOKUP(E$1,dataRowRange,ActualDataRange))</f>
-        <v>CARE</v>
+        <v>Cares</v>
       </c>
       <c r="F4" s="31" t="str" cm="1">
         <f t="array" ref="F4">_xlfn.XLOOKUP($A4,DataColumnRange,_xlfn.XLOOKUP(F$1,dataRowRange,ActualDataRange))</f>
@@ -17987,13 +17997,13 @@
     </row>
     <row r="5" spans="1:39" ht="16" thickBot="1">
       <c r="A5" s="71" t="s">
-        <v>342</v>
+        <v>406</v>
       </c>
       <c r="B5" s="42" t="s">
         <v>310</v>
       </c>
       <c r="C5" s="11" t="s">
-        <v>338</v>
+        <v>402</v>
       </c>
       <c r="D5" s="40" t="str">
         <f>IF(TestCaseConfig!$B$2="Yes","Yes","No")</f>
@@ -18001,7 +18011,7 @@
       </c>
       <c r="E5" s="31" t="str" cm="1">
         <f t="array" ref="E5">_xlfn.XLOOKUP($A5,DataColumnRange,_xlfn.XLOOKUP(E$1,dataRowRange,ActualDataRange))</f>
-        <v>CARE</v>
+        <v>Cares</v>
       </c>
       <c r="F5" s="31" t="str" cm="1">
         <f t="array" ref="F5">_xlfn.XLOOKUP($A5,DataColumnRange,_xlfn.XLOOKUP(F$1,dataRowRange,ActualDataRange))</f>
@@ -18142,13 +18152,13 @@
     </row>
     <row r="6" spans="1:39" ht="16" thickBot="1">
       <c r="A6" s="71" t="s">
-        <v>343</v>
+        <v>407</v>
       </c>
       <c r="B6" s="42" t="s">
         <v>310</v>
       </c>
       <c r="C6" s="11" t="s">
-        <v>338</v>
+        <v>402</v>
       </c>
       <c r="D6" s="40" t="str">
         <f>IF(TestCaseConfig!$B$2="Yes","Yes","No")</f>
@@ -18156,7 +18166,7 @@
       </c>
       <c r="E6" s="31" t="str" cm="1">
         <f t="array" ref="E6">_xlfn.XLOOKUP($A6,DataColumnRange,_xlfn.XLOOKUP(E$1,dataRowRange,ActualDataRange))</f>
-        <v>CARE</v>
+        <v>Cares</v>
       </c>
       <c r="F6" s="31" t="str" cm="1">
         <f t="array" ref="F6">_xlfn.XLOOKUP($A6,DataColumnRange,_xlfn.XLOOKUP(F$1,dataRowRange,ActualDataRange))</f>
@@ -18297,13 +18307,13 @@
     </row>
     <row r="7" spans="1:39" ht="16" thickBot="1">
       <c r="A7" s="71" t="s">
-        <v>344</v>
+        <v>408</v>
       </c>
       <c r="B7" s="42" t="s">
         <v>310</v>
       </c>
       <c r="C7" s="11" t="s">
-        <v>338</v>
+        <v>402</v>
       </c>
       <c r="D7" s="40" t="str">
         <f>IF(TestCaseConfig!$B$2="Yes","Yes","No")</f>
@@ -18311,7 +18321,7 @@
       </c>
       <c r="E7" s="31" t="str" cm="1">
         <f t="array" ref="E7">_xlfn.XLOOKUP($A7,DataColumnRange,_xlfn.XLOOKUP(E$1,dataRowRange,ActualDataRange))</f>
-        <v>CARE</v>
+        <v>Cares</v>
       </c>
       <c r="F7" s="31" t="str" cm="1">
         <f t="array" ref="F7">_xlfn.XLOOKUP($A7,DataColumnRange,_xlfn.XLOOKUP(F$1,dataRowRange,ActualDataRange))</f>
@@ -18976,7 +18986,7 @@
         <v>16</v>
       </c>
       <c r="K2" s="44" t="s">
-        <v>407</v>
+        <v>400</v>
       </c>
       <c r="L2" s="44">
         <v>30</v>
@@ -19088,7 +19098,7 @@
         <v>16</v>
       </c>
       <c r="K3" s="44" t="s">
-        <v>407</v>
+        <v>400</v>
       </c>
       <c r="L3" s="44">
         <v>90</v>
@@ -19200,7 +19210,7 @@
         <v>16</v>
       </c>
       <c r="K4" s="44" t="s">
-        <v>407</v>
+        <v>400</v>
       </c>
       <c r="L4" s="44">
         <v>10</v>
@@ -19312,7 +19322,7 @@
         <v>16</v>
       </c>
       <c r="K5" s="44" t="s">
-        <v>407</v>
+        <v>400</v>
       </c>
       <c r="L5" s="44">
         <v>30</v>
@@ -19424,7 +19434,7 @@
         <v>16</v>
       </c>
       <c r="K6" s="44" t="s">
-        <v>407</v>
+        <v>400</v>
       </c>
       <c r="L6" s="44">
         <v>90</v>
@@ -19536,7 +19546,7 @@
         <v>16</v>
       </c>
       <c r="K7" s="44" t="s">
-        <v>407</v>
+        <v>400</v>
       </c>
       <c r="L7" s="44">
         <v>10</v>
@@ -23680,7 +23690,7 @@
         <v>186</v>
       </c>
       <c r="K44" s="44" t="s">
-        <v>408</v>
+        <v>401</v>
       </c>
       <c r="L44" s="44">
         <v>10</v>
@@ -23792,7 +23802,7 @@
         <v>187</v>
       </c>
       <c r="K45" s="44" t="s">
-        <v>408</v>
+        <v>401</v>
       </c>
       <c r="L45" s="44">
         <v>10</v>
@@ -23904,7 +23914,7 @@
         <v>188</v>
       </c>
       <c r="K46" s="44" t="s">
-        <v>408</v>
+        <v>401</v>
       </c>
       <c r="L46" s="44">
         <v>10</v>
@@ -24016,7 +24026,7 @@
         <v>186</v>
       </c>
       <c r="K47" s="44" t="s">
-        <v>408</v>
+        <v>401</v>
       </c>
       <c r="L47" s="44">
         <v>10</v>
@@ -24128,7 +24138,7 @@
         <v>187</v>
       </c>
       <c r="K48" s="44" t="s">
-        <v>408</v>
+        <v>401</v>
       </c>
       <c r="L48" s="44">
         <v>10</v>
@@ -24240,7 +24250,7 @@
         <v>188</v>
       </c>
       <c r="K49" s="44" t="s">
-        <v>408</v>
+        <v>401</v>
       </c>
       <c r="L49" s="44">
         <v>10</v>
@@ -32568,13 +32578,13 @@
     <row r="124" spans="1:36" s="61" customFormat="1">
       <c r="A124" s="61" t="str">
         <f t="shared" si="1"/>
-        <v>createAndConfirmGuidedBookingHumanRemains_CARE_Adult_Domestic</v>
+        <v>createAndConfirmGuidedBookingHumanRemains_Cares_Adult_Domestic</v>
       </c>
       <c r="B124" s="61" t="s">
         <v>310</v>
       </c>
-      <c r="C124" s="61" t="s">
-        <v>338</v>
+      <c r="C124" s="76" t="s">
+        <v>402</v>
       </c>
       <c r="D124" s="46" t="s">
         <v>125</v>
@@ -32679,13 +32689,13 @@
     <row r="125" spans="1:36" s="61" customFormat="1">
       <c r="A125" s="61" t="str">
         <f t="shared" si="1"/>
-        <v>createAndConfirmGuidedBookingHumanRemains_CARE_ChildInfant_Domestic</v>
+        <v>createAndConfirmGuidedBookingHumanRemains_Cares_ChildInfant_Domestic</v>
       </c>
       <c r="B125" s="61" t="s">
         <v>310</v>
       </c>
-      <c r="C125" s="61" t="s">
-        <v>338</v>
+      <c r="C125" s="76" t="s">
+        <v>402</v>
       </c>
       <c r="D125" s="46" t="s">
         <v>125</v>
@@ -32790,13 +32800,13 @@
     <row r="126" spans="1:36" s="61" customFormat="1">
       <c r="A126" s="61" t="str">
         <f t="shared" si="1"/>
-        <v>createAndConfirmGuidedBookingHumanRemains_CARE_CrematedRemains_Domestic</v>
+        <v>createAndConfirmGuidedBookingHumanRemains_Cares_CrematedRemains_Domestic</v>
       </c>
       <c r="B126" s="61" t="s">
         <v>310</v>
       </c>
-      <c r="C126" s="61" t="s">
-        <v>338</v>
+      <c r="C126" s="76" t="s">
+        <v>402</v>
       </c>
       <c r="D126" s="46" t="s">
         <v>125</v>
@@ -32901,13 +32911,13 @@
     <row r="127" spans="1:36" s="61" customFormat="1">
       <c r="A127" s="61" t="str">
         <f t="shared" si="1"/>
-        <v>createAndConfirmGuidedBookingHumanRemains_CARE_Adult_International</v>
+        <v>createAndConfirmGuidedBookingHumanRemains_Cares_Adult_International</v>
       </c>
       <c r="B127" s="61" t="s">
         <v>310</v>
       </c>
-      <c r="C127" s="61" t="s">
-        <v>338</v>
+      <c r="C127" s="76" t="s">
+        <v>402</v>
       </c>
       <c r="D127" s="46" t="s">
         <v>125</v>
@@ -33012,13 +33022,13 @@
     <row r="128" spans="1:36" s="61" customFormat="1">
       <c r="A128" s="61" t="str">
         <f t="shared" si="1"/>
-        <v>createAndConfirmGuidedBookingHumanRemains_CARE_ChildInfant_International</v>
+        <v>createAndConfirmGuidedBookingHumanRemains_Cares_ChildInfant_International</v>
       </c>
       <c r="B128" s="61" t="s">
         <v>310</v>
       </c>
-      <c r="C128" s="61" t="s">
-        <v>338</v>
+      <c r="C128" s="76" t="s">
+        <v>402</v>
       </c>
       <c r="D128" s="46" t="s">
         <v>125</v>
@@ -33123,13 +33133,13 @@
     <row r="129" spans="1:36" s="61" customFormat="1">
       <c r="A129" s="61" t="str">
         <f t="shared" ref="A129" si="2">_xlfn.CONCAT("createAndConfirmGuidedBooking",SUBSTITUTE(B129," ","_"),"_",SUBSTITUTE(C129," ","_"),"_",SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(J129," ",""),"-",""),"/",""),"–",""),"+",""),"°",""),",",""),"_",SUBSTITUTE(AJ129," ","_"))</f>
-        <v>createAndConfirmGuidedBookingHumanRemains_CARE_CrematedRemains_International</v>
+        <v>createAndConfirmGuidedBookingHumanRemains_Cares_CrematedRemains_International</v>
       </c>
       <c r="B129" s="61" t="s">
         <v>310</v>
       </c>
-      <c r="C129" s="61" t="s">
-        <v>338</v>
+      <c r="C129" s="76" t="s">
+        <v>402</v>
       </c>
       <c r="D129" s="46" t="s">
         <v>125</v>
@@ -33233,7 +33243,7 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:AL129" xr:uid="{1DAEE888-1773-9E47-9558-1F0A440779BF}"/>
-  <phoneticPr fontId="4" type="noConversion"/>
+  <phoneticPr fontId="5" type="noConversion"/>
   <hyperlinks>
     <hyperlink ref="D2" r:id="rId1" xr:uid="{A27DD8EB-70E3-9343-A2F0-4EC1F414F378}"/>
     <hyperlink ref="D3" r:id="rId2" xr:uid="{B7F22B40-D1E3-41A2-B580-43255BDF4D3A}"/>
@@ -33540,7 +33550,7 @@
     </row>
     <row r="2" spans="1:41" ht="16.5" thickBot="1">
       <c r="A2" s="74" t="s">
-        <v>345</v>
+        <v>338</v>
       </c>
       <c r="B2" s="38" t="str" cm="1">
         <f t="array" ref="B2">_xlfn.XLOOKUP($A2,DataColumnRange,_xlfn.XLOOKUP(B$1,dataRowRange,ActualDataRange))</f>
@@ -33703,7 +33713,7 @@
     </row>
     <row r="3" spans="1:41" ht="16.5" thickBot="1">
       <c r="A3" s="75" t="s">
-        <v>346</v>
+        <v>339</v>
       </c>
       <c r="B3" s="38" t="str" cm="1">
         <f t="array" ref="B3">_xlfn.XLOOKUP($A3,DataColumnRange,_xlfn.XLOOKUP(B$1,dataRowRange,ActualDataRange))</f>
@@ -33866,7 +33876,7 @@
     </row>
     <row r="4" spans="1:41" ht="16.5" thickBot="1">
       <c r="A4" s="75" t="s">
-        <v>347</v>
+        <v>340</v>
       </c>
       <c r="B4" s="38" t="str" cm="1">
         <f t="array" ref="B4">_xlfn.XLOOKUP($A4,DataColumnRange,_xlfn.XLOOKUP(B$1,dataRowRange,ActualDataRange))</f>
@@ -34030,7 +34040,7 @@
     </row>
     <row r="5" spans="1:41" ht="16.5" thickBot="1">
       <c r="A5" s="75" t="s">
-        <v>348</v>
+        <v>341</v>
       </c>
       <c r="B5" s="38" t="str" cm="1">
         <f t="array" ref="B5">_xlfn.XLOOKUP($A5,DataColumnRange,_xlfn.XLOOKUP(B$1,dataRowRange,ActualDataRange))</f>
@@ -34194,7 +34204,7 @@
     </row>
     <row r="6" spans="1:41" ht="16.5" thickBot="1">
       <c r="A6" s="75" t="s">
-        <v>349</v>
+        <v>342</v>
       </c>
       <c r="B6" s="38" t="str" cm="1">
         <f t="array" ref="B6">_xlfn.XLOOKUP($A6,DataColumnRange,_xlfn.XLOOKUP(B$1,dataRowRange,ActualDataRange))</f>
@@ -34358,7 +34368,7 @@
     </row>
     <row r="7" spans="1:41" ht="16.5" thickBot="1">
       <c r="A7" s="75" t="s">
-        <v>350</v>
+        <v>343</v>
       </c>
       <c r="B7" s="38" t="str" cm="1">
         <f t="array" ref="B7">_xlfn.XLOOKUP($A7,DataColumnRange,_xlfn.XLOOKUP(B$1,dataRowRange,ActualDataRange))</f>
@@ -34521,7 +34531,7 @@
       </c>
     </row>
   </sheetData>
-  <phoneticPr fontId="4" type="noConversion"/>
+  <phoneticPr fontId="5" type="noConversion"/>
   <hyperlinks>
     <hyperlink ref="D2" location="AdvBkngSTD!A1" display="AdvBkngSTD" xr:uid="{9836EF3A-0C81-384A-B28E-38769E19AD72}"/>
     <hyperlink ref="A1" location="TestCaseConfig!A1" display="TestCases" xr:uid="{B061C974-A2F8-7C4C-A5EC-974E6D31B128}"/>
@@ -34690,7 +34700,7 @@
     </row>
     <row r="2" spans="1:38" ht="17" thickBot="1">
       <c r="A2" s="75" t="s">
-        <v>351</v>
+        <v>344</v>
       </c>
       <c r="B2" s="33" t="s">
         <v>47</v>
@@ -34841,7 +34851,7 @@
     </row>
     <row r="3" spans="1:38" ht="17" thickBot="1">
       <c r="A3" s="75" t="s">
-        <v>352</v>
+        <v>345</v>
       </c>
       <c r="B3" s="33" t="s">
         <v>47</v>
@@ -34992,7 +35002,7 @@
     </row>
     <row r="4" spans="1:38" ht="17" thickBot="1">
       <c r="A4" s="75" t="s">
-        <v>353</v>
+        <v>346</v>
       </c>
       <c r="B4" s="33" t="s">
         <v>47</v>
@@ -35143,7 +35153,7 @@
     </row>
     <row r="5" spans="1:38" ht="17" thickBot="1">
       <c r="A5" s="75" t="s">
-        <v>354</v>
+        <v>347</v>
       </c>
       <c r="B5" s="33" t="s">
         <v>47</v>
@@ -35294,7 +35304,7 @@
     </row>
     <row r="6" spans="1:38" ht="17" thickBot="1">
       <c r="A6" s="75" t="s">
-        <v>355</v>
+        <v>348</v>
       </c>
       <c r="B6" s="33" t="s">
         <v>47</v>
@@ -35445,7 +35455,7 @@
     </row>
     <row r="7" spans="1:38" ht="17" thickBot="1">
       <c r="A7" s="75" t="s">
-        <v>356</v>
+        <v>349</v>
       </c>
       <c r="B7" s="33" t="s">
         <v>47</v>
@@ -35596,7 +35606,7 @@
     </row>
     <row r="8" spans="1:38" ht="17" thickBot="1">
       <c r="A8" s="75" t="s">
-        <v>357</v>
+        <v>350</v>
       </c>
       <c r="B8" s="33" t="s">
         <v>47</v>
@@ -35747,7 +35757,7 @@
     </row>
     <row r="9" spans="1:38" ht="17" thickBot="1">
       <c r="A9" s="75" t="s">
-        <v>358</v>
+        <v>351</v>
       </c>
       <c r="B9" s="33" t="s">
         <v>47</v>
@@ -35898,7 +35908,7 @@
     </row>
     <row r="10" spans="1:38" ht="17" thickBot="1">
       <c r="A10" s="75" t="s">
-        <v>359</v>
+        <v>352</v>
       </c>
       <c r="B10" s="33" t="s">
         <v>47</v>
@@ -36049,7 +36059,7 @@
     </row>
     <row r="11" spans="1:38" ht="17" thickBot="1">
       <c r="A11" s="75" t="s">
-        <v>360</v>
+        <v>353</v>
       </c>
       <c r="B11" s="33" t="s">
         <v>47</v>
@@ -36344,7 +36354,7 @@
     </row>
     <row r="2" spans="1:38" ht="17" thickBot="1">
       <c r="A2" s="75" t="s">
-        <v>361</v>
+        <v>354</v>
       </c>
       <c r="B2" s="33" t="s">
         <v>58</v>
@@ -36495,7 +36505,7 @@
     </row>
     <row r="3" spans="1:38" ht="17" thickBot="1">
       <c r="A3" s="75" t="s">
-        <v>362</v>
+        <v>355</v>
       </c>
       <c r="B3" s="33" t="s">
         <v>58</v>
@@ -36646,7 +36656,7 @@
     </row>
     <row r="4" spans="1:38" ht="17" thickBot="1">
       <c r="A4" s="75" t="s">
-        <v>363</v>
+        <v>356</v>
       </c>
       <c r="B4" s="33" t="s">
         <v>58</v>
@@ -36797,7 +36807,7 @@
     </row>
     <row r="5" spans="1:38" ht="17" thickBot="1">
       <c r="A5" s="75" t="s">
-        <v>364</v>
+        <v>357</v>
       </c>
       <c r="B5" s="33" t="s">
         <v>58</v>
@@ -36948,7 +36958,7 @@
     </row>
     <row r="6" spans="1:38" ht="17" thickBot="1">
       <c r="A6" s="75" t="s">
-        <v>365</v>
+        <v>358</v>
       </c>
       <c r="B6" s="33" t="s">
         <v>58</v>
@@ -37099,7 +37109,7 @@
     </row>
     <row r="7" spans="1:38" ht="17" thickBot="1">
       <c r="A7" s="75" t="s">
-        <v>366</v>
+        <v>359</v>
       </c>
       <c r="B7" s="33" t="s">
         <v>58</v>
@@ -37250,7 +37260,7 @@
     </row>
     <row r="8" spans="1:38" ht="17" thickBot="1">
       <c r="A8" s="75" t="s">
-        <v>367</v>
+        <v>360</v>
       </c>
       <c r="B8" s="33" t="s">
         <v>58</v>
@@ -37401,7 +37411,7 @@
     </row>
     <row r="9" spans="1:38" ht="17" thickBot="1">
       <c r="A9" s="75" t="s">
-        <v>368</v>
+        <v>361</v>
       </c>
       <c r="B9" s="33" t="s">
         <v>58</v>
@@ -37552,7 +37562,7 @@
     </row>
     <row r="10" spans="1:38" ht="17" thickBot="1">
       <c r="A10" s="75" t="s">
-        <v>369</v>
+        <v>362</v>
       </c>
       <c r="B10" s="33" t="s">
         <v>58</v>
@@ -37703,7 +37713,7 @@
     </row>
     <row r="11" spans="1:38" ht="17" thickBot="1">
       <c r="A11" s="75" t="s">
-        <v>370</v>
+        <v>363</v>
       </c>
       <c r="B11" s="33" t="s">
         <v>58</v>
@@ -37996,7 +38006,7 @@
     </row>
     <row r="2" spans="1:38" ht="17" thickBot="1">
       <c r="A2" s="75" t="s">
-        <v>371</v>
+        <v>364</v>
       </c>
       <c r="B2" s="32" t="s">
         <v>44</v>
@@ -38147,7 +38157,7 @@
     </row>
     <row r="3" spans="1:38" ht="17" thickBot="1">
       <c r="A3" s="75" t="s">
-        <v>372</v>
+        <v>365</v>
       </c>
       <c r="B3" s="32" t="s">
         <v>44</v>
@@ -38298,7 +38308,7 @@
     </row>
     <row r="4" spans="1:38" ht="17" thickBot="1">
       <c r="A4" s="75" t="s">
-        <v>373</v>
+        <v>366</v>
       </c>
       <c r="B4" s="32" t="s">
         <v>44</v>
@@ -38449,7 +38459,7 @@
     </row>
     <row r="5" spans="1:38" ht="17" thickBot="1">
       <c r="A5" s="75" t="s">
-        <v>374</v>
+        <v>367</v>
       </c>
       <c r="B5" s="32" t="s">
         <v>44</v>
@@ -38600,7 +38610,7 @@
     </row>
     <row r="6" spans="1:38" ht="17" thickBot="1">
       <c r="A6" s="75" t="s">
-        <v>375</v>
+        <v>368</v>
       </c>
       <c r="B6" s="32" t="s">
         <v>44</v>
@@ -38751,7 +38761,7 @@
     </row>
     <row r="7" spans="1:38" ht="17" thickBot="1">
       <c r="A7" s="75" t="s">
-        <v>376</v>
+        <v>369</v>
       </c>
       <c r="B7" s="32" t="s">
         <v>44</v>
@@ -38902,7 +38912,7 @@
     </row>
     <row r="8" spans="1:38" ht="17" thickBot="1">
       <c r="A8" s="75" t="s">
-        <v>377</v>
+        <v>370</v>
       </c>
       <c r="B8" s="32" t="s">
         <v>44</v>
@@ -39053,7 +39063,7 @@
     </row>
     <row r="9" spans="1:38" ht="17" thickBot="1">
       <c r="A9" s="75" t="s">
-        <v>378</v>
+        <v>371</v>
       </c>
       <c r="B9" s="32" t="s">
         <v>44</v>
@@ -39204,7 +39214,7 @@
     </row>
     <row r="10" spans="1:38" ht="17" thickBot="1">
       <c r="A10" s="75" t="s">
-        <v>379</v>
+        <v>372</v>
       </c>
       <c r="B10" s="32" t="s">
         <v>44</v>
@@ -39355,7 +39365,7 @@
     </row>
     <row r="11" spans="1:38" ht="17" thickBot="1">
       <c r="A11" s="75" t="s">
-        <v>380</v>
+        <v>373</v>
       </c>
       <c r="B11" s="32" t="s">
         <v>44</v>
@@ -39506,7 +39516,7 @@
     </row>
     <row r="12" spans="1:38" ht="17" thickBot="1">
       <c r="A12" s="75" t="s">
-        <v>381</v>
+        <v>374</v>
       </c>
       <c r="B12" s="32" t="s">
         <v>44</v>
@@ -39657,7 +39667,7 @@
     </row>
     <row r="13" spans="1:38" ht="17" thickBot="1">
       <c r="A13" s="75" t="s">
-        <v>382</v>
+        <v>375</v>
       </c>
       <c r="B13" s="32" t="s">
         <v>44</v>
@@ -39951,7 +39961,7 @@
     </row>
     <row r="2" spans="1:38" ht="17" thickBot="1">
       <c r="A2" s="75" t="s">
-        <v>383</v>
+        <v>376</v>
       </c>
       <c r="B2" s="33" t="s">
         <v>87</v>
@@ -40102,7 +40112,7 @@
     </row>
     <row r="3" spans="1:38" ht="17" thickBot="1">
       <c r="A3" s="75" t="s">
-        <v>384</v>
+        <v>377</v>
       </c>
       <c r="B3" s="33" t="s">
         <v>87</v>
@@ -40253,7 +40263,7 @@
     </row>
     <row r="4" spans="1:38" ht="17" thickBot="1">
       <c r="A4" s="75" t="s">
-        <v>385</v>
+        <v>378</v>
       </c>
       <c r="B4" s="33" t="s">
         <v>87</v>
@@ -40404,7 +40414,7 @@
     </row>
     <row r="5" spans="1:38" ht="17" thickBot="1">
       <c r="A5" s="75" t="s">
-        <v>386</v>
+        <v>379</v>
       </c>
       <c r="B5" s="33" t="s">
         <v>87</v>
@@ -40699,7 +40709,7 @@
     </row>
     <row r="2" spans="1:38" ht="17" thickBot="1">
       <c r="A2" s="75" t="s">
-        <v>387</v>
+        <v>380</v>
       </c>
       <c r="B2" s="32" t="s">
         <v>89</v>
@@ -40850,7 +40860,7 @@
     </row>
     <row r="3" spans="1:38" ht="17" thickBot="1">
       <c r="A3" s="75" t="s">
-        <v>388</v>
+        <v>381</v>
       </c>
       <c r="B3" s="32" t="s">
         <v>89</v>
@@ -41001,7 +41011,7 @@
     </row>
     <row r="4" spans="1:38" ht="17" thickBot="1">
       <c r="A4" s="75" t="s">
-        <v>389</v>
+        <v>382</v>
       </c>
       <c r="B4" s="32" t="s">
         <v>89</v>
@@ -41152,7 +41162,7 @@
     </row>
     <row r="5" spans="1:38" ht="17" thickBot="1">
       <c r="A5" s="75" t="s">
-        <v>390</v>
+        <v>383</v>
       </c>
       <c r="B5" s="32" t="s">
         <v>89</v>
@@ -41303,7 +41313,7 @@
     </row>
     <row r="6" spans="1:38" ht="17" thickBot="1">
       <c r="A6" s="75" t="s">
-        <v>391</v>
+        <v>384</v>
       </c>
       <c r="B6" s="32" t="s">
         <v>89</v>
@@ -41454,7 +41464,7 @@
     </row>
     <row r="7" spans="1:38" ht="17" thickBot="1">
       <c r="A7" s="75" t="s">
-        <v>392</v>
+        <v>385</v>
       </c>
       <c r="B7" s="32" t="s">
         <v>89</v>

</xml_diff>